<commit_message>
Finished verbs.xlsx readings for furigana
</commit_message>
<xml_diff>
--- a/verbs.xlsx
+++ b/verbs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BradHunt\Documents\japanese-practice\verbs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24D9CD2-D997-46B2-BFD3-E468FB16F2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4805F6E8-B036-41CB-8C7D-2EF7B1677EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1845" windowWidth="29040" windowHeight="15720" xr2:uid="{9921D540-D520-4E46-B0DA-C77DD5C34F2D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="239">
   <si>
     <t>Dictionary</t>
   </si>
@@ -609,6 +609,150 @@
   </si>
   <si>
     <t>Present - Affirmative - Polite Reading</t>
+  </si>
+  <si>
+    <t>Present - Negative - Polite Reading</t>
+  </si>
+  <si>
+    <t>Past - Affirmative - Polite Reading</t>
+  </si>
+  <si>
+    <t>Past - Negative - Polite Reading</t>
+  </si>
+  <si>
+    <t>Volitional - Polite Reading</t>
+  </si>
+  <si>
+    <t>Desire Reading</t>
+  </si>
+  <si>
+    <t>Negative Stem Reading</t>
+  </si>
+  <si>
+    <t>Present - Negative - Plain Reading</t>
+  </si>
+  <si>
+    <t>Past - Negative - Plain Reading</t>
+  </si>
+  <si>
+    <t>Past - Affirmative - Plain Reading</t>
+  </si>
+  <si>
+    <t>Linking Reading</t>
+  </si>
+  <si>
+    <t>いか</t>
+  </si>
+  <si>
+    <t>のま</t>
+  </si>
+  <si>
+    <t>よま</t>
+  </si>
+  <si>
+    <t>あわ</t>
+  </si>
+  <si>
+    <t>かわ</t>
+  </si>
+  <si>
+    <t>かか</t>
+  </si>
+  <si>
+    <t>とら</t>
+  </si>
+  <si>
+    <t>また</t>
+  </si>
+  <si>
+    <t>わから</t>
+  </si>
+  <si>
+    <t>のら</t>
+  </si>
+  <si>
+    <t>かえら</t>
+  </si>
+  <si>
+    <t>はなさ</t>
+  </si>
+  <si>
+    <t>およが</t>
+  </si>
+  <si>
+    <t>こ</t>
+  </si>
+  <si>
+    <t>きた</t>
+  </si>
+  <si>
+    <t>きて</t>
+  </si>
+  <si>
+    <t>かった</t>
+  </si>
+  <si>
+    <t>のった</t>
+  </si>
+  <si>
+    <t>とった</t>
+  </si>
+  <si>
+    <t>まった</t>
+  </si>
+  <si>
+    <t>わかった</t>
+  </si>
+  <si>
+    <t>いた</t>
+  </si>
+  <si>
+    <t>ねた</t>
+  </si>
+  <si>
+    <t>みた</t>
+  </si>
+  <si>
+    <t>かえった</t>
+  </si>
+  <si>
+    <t>きいた</t>
+  </si>
+  <si>
+    <t>のんだ</t>
+  </si>
+  <si>
+    <t>はなした</t>
+  </si>
+  <si>
+    <t>よんだ</t>
+  </si>
+  <si>
+    <t>かいた</t>
+  </si>
+  <si>
+    <t>およいだ</t>
+  </si>
+  <si>
+    <t>でかけた</t>
+  </si>
+  <si>
+    <t>おきた</t>
+  </si>
+  <si>
+    <t>たべた</t>
+  </si>
+  <si>
+    <t>なかった</t>
+  </si>
+  <si>
+    <t>ない</t>
+  </si>
+  <si>
+    <t>いった</t>
+  </si>
+  <si>
+    <t>いって</t>
   </si>
 </sst>
 </file>
@@ -1069,24 +1213,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{566C2546-B21A-4059-8C0C-B1CB9D497EEB}">
-  <dimension ref="A1:Y25"/>
+  <dimension ref="A1:AH25"/>
   <sheetFormatPr defaultRowHeight="17.5" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" style="7" customWidth="1"/>
-    <col min="2" max="3" width="24.6328125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="24.6328125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="18.6328125" style="6" customWidth="1"/>
-    <col min="7" max="7" width="24.6328125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="33.6328125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="42.6328125" style="6" customWidth="1"/>
-    <col min="10" max="14" width="33.6328125" style="6" customWidth="1"/>
-    <col min="15" max="15" width="18.6328125" style="6" customWidth="1"/>
-    <col min="16" max="19" width="33.6328125" style="6" customWidth="1"/>
-    <col min="20" max="25" width="8.7265625" style="6"/>
+    <col min="1" max="1" width="12.26953125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.08984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="42.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="38.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="36.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="29.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="39" style="6" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.6328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="35.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="38" style="6" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="30" max="34" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1118,34 +1280,64 @@
         <v>6</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="S1" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="T1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="U1" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="V1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="W1" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="X1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="Y1" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="Z1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="AB1" s="5" t="s">
         <v>15</v>
       </c>
+      <c r="AC1" s="5" t="s">
+        <v>200</v>
+      </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A2" s="7" t="s">
         <v>16</v>
       </c>
@@ -1180,40 +1372,77 @@
         <v>行きません</v>
       </c>
       <c r="K2" s="7" t="str">
+        <f>_xlfn.CONCAT(G2,"ません")</f>
+        <v>いきません</v>
+      </c>
+      <c r="L2" s="7" t="str">
         <f>_xlfn.CONCAT(F2,"ました")</f>
         <v>行きました</v>
       </c>
-      <c r="L2" s="7" t="str">
+      <c r="M2" s="7" t="str">
+        <f>_xlfn.CONCAT(G2,"ました")</f>
+        <v>いきました</v>
+      </c>
+      <c r="N2" s="7" t="str">
         <f>_xlfn.CONCAT(F2,"ませんでした")</f>
         <v>行きませんでした</v>
       </c>
-      <c r="M2" s="7" t="str">
+      <c r="O2" s="7" t="str">
+        <f>_xlfn.CONCAT(G2,"ませんでした")</f>
+        <v>いきませんでした</v>
+      </c>
+      <c r="P2" s="7" t="str">
         <f>_xlfn.CONCAT(F2,"ましょう")</f>
         <v>行きましょう</v>
       </c>
-      <c r="N2" s="7" t="str">
+      <c r="Q2" s="7" t="str">
+        <f>_xlfn.CONCAT(G2,"ましょう")</f>
+        <v>いきましょう</v>
+      </c>
+      <c r="R2" s="7" t="str">
         <f>_xlfn.CONCAT(F2,"たい")</f>
         <v>行きたい</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="S2" s="7" t="str">
+        <f>_xlfn.CONCAT(G2,"たい")</f>
+        <v>いきたい</v>
+      </c>
+      <c r="T2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="7" t="str">
-        <f>_xlfn.CONCAT(O2,"ない")</f>
+      <c r="U2" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="V2" s="7" t="str">
+        <f>_xlfn.CONCAT(T2,"ない")</f>
         <v>行かない</v>
       </c>
-      <c r="Q2" s="7" t="str">
-        <f>_xlfn.CONCAT(O2,"なかった")</f>
+      <c r="W2" s="7" t="str">
+        <f>_xlfn.CONCAT(U2,"ない")</f>
+        <v>いかない</v>
+      </c>
+      <c r="X2" s="7" t="str">
+        <f>_xlfn.CONCAT(T2,"なかった")</f>
         <v>行かなかった</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="Y2" s="7" t="str">
+        <f>_xlfn.CONCAT(U2,"なかった")</f>
+        <v>いかなかった</v>
+      </c>
+      <c r="Z2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="AA2" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="AB2" s="8" t="s">
         <v>23</v>
       </c>
+      <c r="AC2" s="8" t="s">
+        <v>238</v>
+      </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A3" s="7" t="s">
         <v>24</v>
       </c>
@@ -1248,40 +1477,78 @@
         <v>帰りません</v>
       </c>
       <c r="K3" s="7" t="str">
-        <f t="shared" ref="K3:K25" si="3">_xlfn.CONCAT(F3,"ました")</f>
+        <f t="shared" ref="K3:K25" si="3">_xlfn.CONCAT(G3,"ません")</f>
+        <v>かえりません</v>
+      </c>
+      <c r="L3" s="7" t="str">
+        <f t="shared" ref="L3:L25" si="4">_xlfn.CONCAT(F3,"ました")</f>
         <v>帰りました</v>
       </c>
-      <c r="L3" s="7" t="str">
-        <f t="shared" ref="L3:L25" si="4">_xlfn.CONCAT(F3,"ませんでした")</f>
+      <c r="M3" s="7" t="str">
+        <f t="shared" ref="M3:M25" si="5">_xlfn.CONCAT(G3,"ました")</f>
+        <v>かえりました</v>
+      </c>
+      <c r="N3" s="7" t="str">
+        <f t="shared" ref="N3:N25" si="6">_xlfn.CONCAT(F3,"ませんでした")</f>
         <v>帰りませんでした</v>
       </c>
-      <c r="M3" s="7" t="str">
-        <f t="shared" ref="M3:M25" si="5">_xlfn.CONCAT(F3,"ましょう")</f>
+      <c r="O3" s="7" t="str">
+        <f t="shared" ref="O3:O25" si="7">_xlfn.CONCAT(G3,"ませんでした")</f>
+        <v>かえりませんでした</v>
+      </c>
+      <c r="P3" s="7" t="str">
+        <f t="shared" ref="P3:P25" si="8">_xlfn.CONCAT(F3,"ましょう")</f>
         <v>帰りましょう</v>
       </c>
-      <c r="N3" s="7" t="str">
-        <f t="shared" ref="N3:N25" si="6">_xlfn.CONCAT(F3,"たい")</f>
+      <c r="Q3" s="7" t="str">
+        <f t="shared" ref="Q3:Q25" si="9">_xlfn.CONCAT(G3,"ましょう")</f>
+        <v>かえりましょう</v>
+      </c>
+      <c r="R3" s="7" t="str">
+        <f t="shared" ref="R3:R25" si="10">_xlfn.CONCAT(F3,"たい")</f>
         <v>帰りたい</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="S3" s="7" t="str">
+        <f t="shared" ref="S3:S25" si="11">_xlfn.CONCAT(G3,"たい")</f>
+        <v>かえりたい</v>
+      </c>
+      <c r="T3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="P3" s="7" t="str">
-        <f t="shared" ref="P3:P25" si="7">_xlfn.CONCAT(O3,"ない")</f>
+      <c r="U3" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="V3" s="7" t="str">
+        <f t="shared" ref="V3:W25" si="12">_xlfn.CONCAT(T3,"ない")</f>
         <v>帰らない</v>
       </c>
-      <c r="Q3" s="7" t="str">
-        <f t="shared" ref="Q3:Q8" si="8">_xlfn.CONCAT(O3,"なかった")</f>
+      <c r="W3" s="7" t="str">
+        <f t="shared" ref="W3:W8" si="13">_xlfn.CONCAT(U3,"ない")</f>
+        <v>かえらない</v>
+      </c>
+      <c r="X3" s="7" t="str">
+        <f t="shared" ref="X3:X8" si="14">_xlfn.CONCAT(T3,"なかった")</f>
         <v>帰らなかった</v>
       </c>
-      <c r="R3" s="7" t="s">
+      <c r="Y3" s="7" t="str">
+        <f t="shared" ref="Y3:Y8" si="15">_xlfn.CONCAT(U3,"なかった")</f>
+        <v>かえらなかった</v>
+      </c>
+      <c r="Z3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="AA3" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB3" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="AC3" s="7" t="str">
+        <f>LEFT(AA3,LEN(AA3)-1) &amp; "て"</f>
+        <v>かえって</v>
+      </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A4" s="7" t="s">
         <v>31</v>
       </c>
@@ -1317,39 +1584,77 @@
       </c>
       <c r="K4" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>聞きました</v>
+        <v>ききません</v>
       </c>
       <c r="L4" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>聞きませんでした</v>
+        <v>聞きました</v>
       </c>
       <c r="M4" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>聞きましょう</v>
+        <v>ききました</v>
       </c>
       <c r="N4" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>聞きませんでした</v>
+      </c>
+      <c r="O4" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>ききませんでした</v>
+      </c>
+      <c r="P4" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>聞きましょう</v>
+      </c>
+      <c r="Q4" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>ききましょう</v>
+      </c>
+      <c r="R4" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>聞きたい</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="S4" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>ききたい</v>
+      </c>
+      <c r="T4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="P4" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U4" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="V4" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>聞かない</v>
       </c>
-      <c r="Q4" s="7" t="str">
-        <f t="shared" si="8"/>
+      <c r="W4" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>かかない</v>
+      </c>
+      <c r="X4" s="7" t="str">
+        <f t="shared" si="14"/>
         <v>聞かなかった</v>
       </c>
-      <c r="R4" s="7" t="s">
+      <c r="Y4" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>かかなかった</v>
+      </c>
+      <c r="Z4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="S4" s="7" t="s">
+      <c r="AA4" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB4" s="7" t="s">
         <v>36</v>
       </c>
+      <c r="AC4" s="7" t="str">
+        <f t="shared" ref="AC4:AC23" si="16">LEFT(AA4,LEN(AA4)-1) &amp; "て"</f>
+        <v>きいて</v>
+      </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A5" s="7" t="s">
         <v>37</v>
       </c>
@@ -1385,39 +1690,77 @@
       </c>
       <c r="K5" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>飲みました</v>
+        <v>のみません</v>
       </c>
       <c r="L5" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>飲みませんでした</v>
+        <v>飲みました</v>
       </c>
       <c r="M5" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>飲みましょう</v>
+        <v>のみました</v>
       </c>
       <c r="N5" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>飲みませんでした</v>
+      </c>
+      <c r="O5" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>のみませんでした</v>
+      </c>
+      <c r="P5" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>飲みましょう</v>
+      </c>
+      <c r="Q5" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>のみましょう</v>
+      </c>
+      <c r="R5" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>飲みたい</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="S5" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>のみたい</v>
+      </c>
+      <c r="T5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="P5" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U5" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="V5" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>飲まない</v>
       </c>
-      <c r="Q5" s="7" t="str">
-        <f t="shared" si="8"/>
+      <c r="W5" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>のまない</v>
+      </c>
+      <c r="X5" s="7" t="str">
+        <f t="shared" si="14"/>
         <v>飲まなかった</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="Y5" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>のまなかった</v>
+      </c>
+      <c r="Z5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="S5" s="7" t="s">
+      <c r="AA5" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB5" s="7" t="s">
         <v>42</v>
       </c>
+      <c r="AC5" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>のんて</v>
+      </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A6" s="7" t="s">
         <v>43</v>
       </c>
@@ -1453,39 +1796,77 @@
       </c>
       <c r="K6" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>話しました</v>
+        <v>はなしません</v>
       </c>
       <c r="L6" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>話しませんでした</v>
+        <v>話しました</v>
       </c>
       <c r="M6" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>話しましょう</v>
+        <v>はなしました</v>
       </c>
       <c r="N6" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>話しませんでした</v>
+      </c>
+      <c r="O6" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>はなしませんでした</v>
+      </c>
+      <c r="P6" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>話しましょう</v>
+      </c>
+      <c r="Q6" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>はなしましょう</v>
+      </c>
+      <c r="R6" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>話したい</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="S6" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>はなしたい</v>
+      </c>
+      <c r="T6" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U6" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="V6" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>話さない</v>
       </c>
-      <c r="Q6" s="7" t="str">
-        <f t="shared" si="8"/>
+      <c r="W6" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>はなさない</v>
+      </c>
+      <c r="X6" s="7" t="str">
+        <f t="shared" si="14"/>
         <v>話さなかった</v>
       </c>
-      <c r="R6" s="7" t="s">
+      <c r="Y6" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>はなさなかった</v>
+      </c>
+      <c r="Z6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="S6" s="7" t="s">
+      <c r="AA6" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="AB6" s="7" t="s">
         <v>48</v>
       </c>
+      <c r="AC6" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>はなして</v>
+      </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A7" s="7" t="s">
         <v>49</v>
       </c>
@@ -1521,39 +1902,77 @@
       </c>
       <c r="K7" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>読みました</v>
+        <v>よみません</v>
       </c>
       <c r="L7" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>読みませんでした</v>
+        <v>読みました</v>
       </c>
       <c r="M7" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>読みましょう</v>
+        <v>よみました</v>
       </c>
       <c r="N7" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>読みませんでした</v>
+      </c>
+      <c r="O7" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>よみませんでした</v>
+      </c>
+      <c r="P7" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>読みましょう</v>
+      </c>
+      <c r="Q7" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>よみましょう</v>
+      </c>
+      <c r="R7" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>読みたい</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="S7" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>よみたい</v>
+      </c>
+      <c r="T7" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="P7" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U7" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="V7" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>読まない</v>
       </c>
-      <c r="Q7" s="7" t="str">
-        <f t="shared" si="8"/>
+      <c r="W7" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>よまない</v>
+      </c>
+      <c r="X7" s="7" t="str">
+        <f t="shared" si="14"/>
         <v>読まなかった</v>
       </c>
-      <c r="R7" s="7" t="s">
+      <c r="Y7" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>よまなかった</v>
+      </c>
+      <c r="Z7" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="S7" s="7" t="s">
+      <c r="AA7" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB7" s="7" t="s">
         <v>54</v>
       </c>
+      <c r="AC7" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>よんて</v>
+      </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A8" s="7" t="s">
         <v>55</v>
       </c>
@@ -1589,39 +2008,77 @@
       </c>
       <c r="K8" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>会いました</v>
+        <v>あいません</v>
       </c>
       <c r="L8" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>会いませんでした</v>
+        <v>会いました</v>
       </c>
       <c r="M8" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>会いましょう</v>
+        <v>あいました</v>
       </c>
       <c r="N8" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>会いませんでした</v>
+      </c>
+      <c r="O8" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>あいませんでした</v>
+      </c>
+      <c r="P8" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>会いましょう</v>
+      </c>
+      <c r="Q8" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>あいましょう</v>
+      </c>
+      <c r="R8" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>会いたい</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="S8" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>あいたい</v>
+      </c>
+      <c r="T8" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="P8" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U8" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="V8" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>会わない</v>
       </c>
-      <c r="Q8" s="7" t="str">
-        <f t="shared" si="8"/>
+      <c r="W8" s="7" t="str">
+        <f t="shared" si="13"/>
+        <v>あわない</v>
+      </c>
+      <c r="X8" s="7" t="str">
+        <f t="shared" si="14"/>
         <v>会わなかった</v>
       </c>
-      <c r="R8" s="7" t="s">
+      <c r="Y8" s="7" t="str">
+        <f t="shared" si="15"/>
+        <v>あわなかった</v>
+      </c>
+      <c r="Z8" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="S8" s="7" t="s">
+      <c r="AA8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB8" s="7" t="s">
         <v>60</v>
       </c>
+      <c r="AC8" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>あって</v>
+      </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A9" s="7" t="s">
         <v>61</v>
       </c>
@@ -1657,37 +2114,73 @@
       </c>
       <c r="K9" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>ありました</v>
+        <v>ありません</v>
       </c>
       <c r="L9" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>ありませんでした</v>
+        <v>ありました</v>
       </c>
       <c r="M9" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>ありましょう</v>
+        <v>ありました</v>
       </c>
       <c r="N9" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>ありませんでした</v>
+      </c>
+      <c r="O9" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>ありませんでした</v>
+      </c>
+      <c r="P9" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>ありましょう</v>
+      </c>
+      <c r="Q9" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>ありましょう</v>
+      </c>
+      <c r="R9" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>ありたい</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="S9" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>ありたい</v>
+      </c>
+      <c r="T9" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="U9" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="V9" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="Q9" s="8" t="s">
+      <c r="W9" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="X9" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="R9" s="7" t="s">
+      <c r="Y9" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="S9" s="7" t="s">
+      <c r="AA9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB9" s="7" t="s">
         <v>68</v>
       </c>
+      <c r="AC9" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>あって</v>
+      </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A10" s="7" t="s">
         <v>69</v>
       </c>
@@ -1723,39 +2216,77 @@
       </c>
       <c r="K10" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>買いました</v>
+        <v>かいません</v>
       </c>
       <c r="L10" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>買いませんでした</v>
+        <v>買いました</v>
       </c>
       <c r="M10" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>買いましょう</v>
+        <v>かいました</v>
       </c>
       <c r="N10" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>買いませんでした</v>
+      </c>
+      <c r="O10" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>かいませんでした</v>
+      </c>
+      <c r="P10" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>買いましょう</v>
+      </c>
+      <c r="Q10" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>かいましょう</v>
+      </c>
+      <c r="R10" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>買いたい</v>
       </c>
-      <c r="O10" s="7" t="s">
+      <c r="S10" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>かいたい</v>
+      </c>
+      <c r="T10" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="P10" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U10" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="V10" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>買わない</v>
       </c>
-      <c r="Q10" s="7" t="str">
-        <f>_xlfn.CONCAT(O10,"なかった")</f>
+      <c r="W10" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>かわない</v>
+      </c>
+      <c r="X10" s="7" t="str">
+        <f>_xlfn.CONCAT(T10,"なかった")</f>
         <v>買わなかった</v>
       </c>
-      <c r="R10" s="7" t="s">
+      <c r="Y10" s="7" t="str">
+        <f>_xlfn.CONCAT(U10,"なかった")</f>
+        <v>かわなかった</v>
+      </c>
+      <c r="Z10" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="S10" s="7" t="s">
+      <c r="AA10" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="AB10" s="7" t="s">
         <v>74</v>
       </c>
+      <c r="AC10" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>かって</v>
+      </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A11" s="7" t="s">
         <v>75</v>
       </c>
@@ -1791,39 +2322,77 @@
       </c>
       <c r="K11" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>書きました</v>
+        <v>かきません</v>
       </c>
       <c r="L11" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>書きませんでした</v>
+        <v>書きました</v>
       </c>
       <c r="M11" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>書きましょう</v>
+        <v>かきました</v>
       </c>
       <c r="N11" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>書きませんでした</v>
+      </c>
+      <c r="O11" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>かきませんでした</v>
+      </c>
+      <c r="P11" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>書きましょう</v>
+      </c>
+      <c r="Q11" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>かきましょう</v>
+      </c>
+      <c r="R11" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>書きたい</v>
       </c>
-      <c r="O11" s="7" t="s">
+      <c r="S11" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>かきたい</v>
+      </c>
+      <c r="T11" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="P11" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U11" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="V11" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>書かない</v>
       </c>
-      <c r="Q11" s="7" t="str">
-        <f t="shared" ref="Q11:Q24" si="9">_xlfn.CONCAT(O11,"なかった")</f>
+      <c r="W11" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>かかない</v>
+      </c>
+      <c r="X11" s="7" t="str">
+        <f t="shared" ref="X11:X24" si="17">_xlfn.CONCAT(T11,"なかった")</f>
         <v>書かなかった</v>
       </c>
-      <c r="R11" s="7" t="s">
+      <c r="Y11" s="7" t="str">
+        <f t="shared" ref="Y11:Y25" si="18">_xlfn.CONCAT(U11,"なかった")</f>
+        <v>かかなかった</v>
+      </c>
+      <c r="Z11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="S11" s="7" t="s">
+      <c r="AA11" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="AB11" s="7" t="s">
         <v>80</v>
       </c>
+      <c r="AC11" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>かいて</v>
+      </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A12" s="7" t="s">
         <v>81</v>
       </c>
@@ -1859,39 +2428,77 @@
       </c>
       <c r="K12" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>撮りました</v>
+        <v>とりません</v>
       </c>
       <c r="L12" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>撮りませんでした</v>
+        <v>撮りました</v>
       </c>
       <c r="M12" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>撮りましょう</v>
+        <v>とりました</v>
       </c>
       <c r="N12" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>撮りたい</v>
-      </c>
-      <c r="O12" s="7" t="s">
-        <v>84</v>
+        <v>撮りませんでした</v>
+      </c>
+      <c r="O12" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>とりませんでした</v>
       </c>
       <c r="P12" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>撮らない</v>
+        <f t="shared" si="8"/>
+        <v>撮りましょう</v>
       </c>
       <c r="Q12" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>とりましょう</v>
+      </c>
+      <c r="R12" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>撮りたい</v>
+      </c>
+      <c r="S12" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>とりたい</v>
+      </c>
+      <c r="T12" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="U12" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="V12" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>撮らない</v>
+      </c>
+      <c r="W12" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>とらない</v>
+      </c>
+      <c r="X12" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>撮らなかった</v>
       </c>
-      <c r="R12" s="7" t="s">
+      <c r="Y12" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>とらなかった</v>
+      </c>
+      <c r="Z12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="S12" s="7" t="s">
+      <c r="AA12" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB12" s="7" t="s">
         <v>86</v>
       </c>
+      <c r="AC12" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>とって</v>
+      </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A13" s="7" t="s">
         <v>87</v>
       </c>
@@ -1927,39 +2534,77 @@
       </c>
       <c r="K13" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>待ちました</v>
+        <v>まちません</v>
       </c>
       <c r="L13" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>待ちませんでした</v>
+        <v>待ちました</v>
       </c>
       <c r="M13" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>待ちましょう</v>
+        <v>まちました</v>
       </c>
       <c r="N13" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>待ちたい</v>
-      </c>
-      <c r="O13" s="7" t="s">
-        <v>90</v>
+        <v>待ちませんでした</v>
+      </c>
+      <c r="O13" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>まちませんでした</v>
       </c>
       <c r="P13" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>待たない</v>
+        <f t="shared" si="8"/>
+        <v>待ちましょう</v>
       </c>
       <c r="Q13" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>まちましょう</v>
+      </c>
+      <c r="R13" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>待ちたい</v>
+      </c>
+      <c r="S13" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>まちたい</v>
+      </c>
+      <c r="T13" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="V13" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>待たない</v>
+      </c>
+      <c r="W13" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>またない</v>
+      </c>
+      <c r="X13" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>待たなかった</v>
       </c>
-      <c r="R13" s="7" t="s">
+      <c r="Y13" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>またなかった</v>
+      </c>
+      <c r="Z13" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="S13" s="7" t="s">
+      <c r="AA13" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="AB13" s="7" t="s">
         <v>92</v>
       </c>
+      <c r="AC13" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>まって</v>
+      </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A14" s="7" t="s">
         <v>93</v>
       </c>
@@ -1995,39 +2640,77 @@
       </c>
       <c r="K14" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>分かりました</v>
+        <v>わかりません</v>
       </c>
       <c r="L14" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>分かりませんでした</v>
+        <v>分かりました</v>
       </c>
       <c r="M14" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>分かりましょう</v>
+        <v>わかりました</v>
       </c>
       <c r="N14" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>分かりたい</v>
-      </c>
-      <c r="O14" s="7" t="s">
-        <v>96</v>
+        <v>分かりませんでした</v>
+      </c>
+      <c r="O14" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>わかりませんでした</v>
       </c>
       <c r="P14" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>分からない</v>
+        <f t="shared" si="8"/>
+        <v>分かりましょう</v>
       </c>
       <c r="Q14" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>わかりましょう</v>
+      </c>
+      <c r="R14" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>分かりたい</v>
+      </c>
+      <c r="S14" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>わかりたい</v>
+      </c>
+      <c r="T14" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="V14" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>分からない</v>
+      </c>
+      <c r="W14" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>わからない</v>
+      </c>
+      <c r="X14" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>分からなかった</v>
       </c>
-      <c r="R14" s="7" t="s">
+      <c r="Y14" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>わからなかった</v>
+      </c>
+      <c r="Z14" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="S14" s="7" t="s">
+      <c r="AA14" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="AB14" s="7" t="s">
         <v>98</v>
       </c>
+      <c r="AC14" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>わかって</v>
+      </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A15" s="7" t="s">
         <v>99</v>
       </c>
@@ -2063,39 +2746,77 @@
       </c>
       <c r="K15" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>泳ぎました</v>
+        <v>およぎません</v>
       </c>
       <c r="L15" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>泳ぎませんでした</v>
+        <v>泳ぎました</v>
       </c>
       <c r="M15" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>泳ぎましょう</v>
+        <v>およぎました</v>
       </c>
       <c r="N15" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>泳ぎたい</v>
-      </c>
-      <c r="O15" s="7" t="s">
-        <v>102</v>
+        <v>泳ぎませんでした</v>
+      </c>
+      <c r="O15" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>およぎませんでした</v>
       </c>
       <c r="P15" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>泳がない</v>
+        <f t="shared" si="8"/>
+        <v>泳ぎましょう</v>
       </c>
       <c r="Q15" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>およぎましょう</v>
+      </c>
+      <c r="R15" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>泳ぎたい</v>
+      </c>
+      <c r="S15" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>およぎたい</v>
+      </c>
+      <c r="T15" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="V15" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>泳がない</v>
+      </c>
+      <c r="W15" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>およがない</v>
+      </c>
+      <c r="X15" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>泳がなかった</v>
       </c>
-      <c r="R15" s="7" t="s">
+      <c r="Y15" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>およがなかった</v>
+      </c>
+      <c r="Z15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="S15" s="7" t="s">
+      <c r="AA15" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB15" s="7" t="s">
         <v>104</v>
       </c>
+      <c r="AC15" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>およいて</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A16" s="7" t="s">
         <v>105</v>
       </c>
@@ -2131,39 +2852,77 @@
       </c>
       <c r="K16" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>乗りました</v>
+        <v>のりません</v>
       </c>
       <c r="L16" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>乗りませんでした</v>
+        <v>乗りました</v>
       </c>
       <c r="M16" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>乗りましょう</v>
+        <v>のりました</v>
       </c>
       <c r="N16" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>乗りたい</v>
-      </c>
-      <c r="O16" s="7" t="s">
-        <v>108</v>
+        <v>乗りませんでした</v>
+      </c>
+      <c r="O16" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>のりませんでした</v>
       </c>
       <c r="P16" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>乗らない</v>
+        <f t="shared" si="8"/>
+        <v>乗りましょう</v>
       </c>
       <c r="Q16" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>のりましょう</v>
+      </c>
+      <c r="R16" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>乗りたい</v>
+      </c>
+      <c r="S16" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>のりたい</v>
+      </c>
+      <c r="T16" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="U16" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="V16" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>乗らない</v>
+      </c>
+      <c r="W16" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>のらない</v>
+      </c>
+      <c r="X16" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>乗らなかった</v>
       </c>
-      <c r="R16" s="7" t="s">
+      <c r="Y16" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>のらなかった</v>
+      </c>
+      <c r="Z16" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="S16" s="7" t="s">
+      <c r="AA16" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB16" s="7" t="s">
         <v>110</v>
       </c>
+      <c r="AC16" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>のって</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A17" s="7" t="s">
         <v>111</v>
       </c>
@@ -2199,39 +2958,77 @@
       </c>
       <c r="K17" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>やりました</v>
+        <v>やりません</v>
       </c>
       <c r="L17" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>やりませんでした</v>
+        <v>やりました</v>
       </c>
       <c r="M17" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>やりましょう</v>
+        <v>やりました</v>
       </c>
       <c r="N17" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>やりたい</v>
-      </c>
-      <c r="O17" s="7" t="s">
-        <v>114</v>
+        <v>やりませんでした</v>
+      </c>
+      <c r="O17" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>やりませんでした</v>
       </c>
       <c r="P17" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>やらない</v>
+        <f t="shared" si="8"/>
+        <v>やりましょう</v>
       </c>
       <c r="Q17" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>やりましょう</v>
+      </c>
+      <c r="R17" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>やりたい</v>
+      </c>
+      <c r="S17" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>やりたい</v>
+      </c>
+      <c r="T17" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="V17" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>やらない</v>
+      </c>
+      <c r="W17" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>やらない</v>
+      </c>
+      <c r="X17" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>やらなかった</v>
       </c>
-      <c r="R17" s="7" t="s">
+      <c r="Y17" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>やらなかった</v>
+      </c>
+      <c r="Z17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="S17" s="7" t="s">
+      <c r="AA17" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB17" s="7" t="s">
         <v>116</v>
       </c>
+      <c r="AC17" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>やって</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A18" s="7" t="s">
         <v>117</v>
       </c>
@@ -2267,41 +3064,80 @@
       </c>
       <c r="K18" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>出かけました</v>
+        <v>でかけません</v>
       </c>
       <c r="L18" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>出かけませんでした</v>
+        <v>出かけました</v>
       </c>
       <c r="M18" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>出かけましょう</v>
+        <v>でかけました</v>
       </c>
       <c r="N18" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>出かけたい</v>
-      </c>
-      <c r="O18" s="7" t="s">
-        <v>121</v>
+        <v>出かけませんでした</v>
+      </c>
+      <c r="O18" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>でかけませんでした</v>
       </c>
       <c r="P18" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>出かけない</v>
+        <f t="shared" si="8"/>
+        <v>出かけましょう</v>
       </c>
       <c r="Q18" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>でかけましょう</v>
+      </c>
+      <c r="R18" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>出かけたい</v>
+      </c>
+      <c r="S18" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>でかけたい</v>
+      </c>
+      <c r="T18" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="U18" s="7" t="str">
+        <f>G18</f>
+        <v>でかけ</v>
+      </c>
+      <c r="V18" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>出かけない</v>
+      </c>
+      <c r="W18" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>でかけない</v>
+      </c>
+      <c r="X18" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>出かけなかった</v>
       </c>
-      <c r="R18" s="7" t="str">
+      <c r="Y18" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>でかけなかった</v>
+      </c>
+      <c r="Z18" s="7" t="str">
         <f>_xlfn.CONCAT(F18,"た")</f>
         <v>出かけた</v>
       </c>
-      <c r="S18" s="7" t="str">
+      <c r="AA18" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB18" s="7" t="str">
         <f>_xlfn.CONCAT(F18,"て")</f>
         <v>出かけて</v>
       </c>
+      <c r="AC18" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>でかけて</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A19" s="7" t="s">
         <v>122</v>
       </c>
@@ -2337,41 +3173,80 @@
       </c>
       <c r="K19" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>いました</v>
+        <v>いません</v>
       </c>
       <c r="L19" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>いませんでした</v>
+        <v>いました</v>
       </c>
       <c r="M19" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>いましょう</v>
+        <v>いました</v>
       </c>
       <c r="N19" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>いたい</v>
-      </c>
-      <c r="O19" s="7" t="s">
-        <v>124</v>
+        <v>いませんでした</v>
+      </c>
+      <c r="O19" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>いませんでした</v>
       </c>
       <c r="P19" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>いない</v>
+        <f t="shared" si="8"/>
+        <v>いましょう</v>
       </c>
       <c r="Q19" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>いましょう</v>
+      </c>
+      <c r="R19" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>いたい</v>
+      </c>
+      <c r="S19" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>いたい</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="U19" s="7" t="str">
+        <f t="shared" ref="U19:U23" si="19">G19</f>
+        <v>い</v>
+      </c>
+      <c r="V19" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>いない</v>
+      </c>
+      <c r="W19" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>いない</v>
+      </c>
+      <c r="X19" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>いなかった</v>
       </c>
-      <c r="R19" s="7" t="str">
-        <f t="shared" ref="R19:R23" si="10">_xlfn.CONCAT(F19,"た")</f>
+      <c r="Y19" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>いなかった</v>
+      </c>
+      <c r="Z19" s="7" t="str">
+        <f t="shared" ref="Z19:Z23" si="20">_xlfn.CONCAT(F19,"た")</f>
         <v>いた</v>
       </c>
-      <c r="S19" s="7" t="str">
-        <f t="shared" ref="S19:S23" si="11">_xlfn.CONCAT(F19,"て")</f>
+      <c r="AA19" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="AB19" s="7" t="str">
+        <f t="shared" ref="AB19:AB23" si="21">_xlfn.CONCAT(F19,"て")</f>
         <v>いて</v>
       </c>
+      <c r="AC19" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>いて</v>
+      </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A20" s="7" t="s">
         <v>125</v>
       </c>
@@ -2407,41 +3282,80 @@
       </c>
       <c r="K20" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>起きました</v>
+        <v>おきません</v>
       </c>
       <c r="L20" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>起きませんでした</v>
+        <v>起きました</v>
       </c>
       <c r="M20" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>起きましょう</v>
+        <v>おきました</v>
       </c>
       <c r="N20" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>起きたい</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>127</v>
+        <v>起きませんでした</v>
+      </c>
+      <c r="O20" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>おきませんでした</v>
       </c>
       <c r="P20" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>起きない</v>
+        <f t="shared" si="8"/>
+        <v>起きましょう</v>
       </c>
       <c r="Q20" s="7" t="str">
         <f t="shared" si="9"/>
-        <v>起きなかった</v>
+        <v>おきましょう</v>
       </c>
       <c r="R20" s="7" t="str">
         <f t="shared" si="10"/>
-        <v>起きた</v>
+        <v>起きたい</v>
       </c>
       <c r="S20" s="7" t="str">
         <f t="shared" si="11"/>
+        <v>おきたい</v>
+      </c>
+      <c r="T20" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="U20" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>おき</v>
+      </c>
+      <c r="V20" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>起きない</v>
+      </c>
+      <c r="W20" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>おきない</v>
+      </c>
+      <c r="X20" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>起きなかった</v>
+      </c>
+      <c r="Y20" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>おきなかった</v>
+      </c>
+      <c r="Z20" s="7" t="str">
+        <f t="shared" si="20"/>
+        <v>起きた</v>
+      </c>
+      <c r="AA20" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB20" s="7" t="str">
+        <f t="shared" si="21"/>
         <v>起きて</v>
       </c>
+      <c r="AC20" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>おきて</v>
+      </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A21" s="7" t="s">
         <v>128</v>
       </c>
@@ -2477,41 +3391,80 @@
       </c>
       <c r="K21" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>食べました</v>
+        <v>たべません</v>
       </c>
       <c r="L21" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>食べませんでした</v>
+        <v>食べました</v>
       </c>
       <c r="M21" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>食べましょう</v>
+        <v>たべました</v>
       </c>
       <c r="N21" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>食べたい</v>
-      </c>
-      <c r="O21" s="7" t="s">
-        <v>130</v>
+        <v>食べませんでした</v>
+      </c>
+      <c r="O21" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>たべませんでした</v>
       </c>
       <c r="P21" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>食べない</v>
+        <f t="shared" si="8"/>
+        <v>食べましょう</v>
       </c>
       <c r="Q21" s="7" t="str">
         <f t="shared" si="9"/>
-        <v>食べなかった</v>
+        <v>たべましょう</v>
       </c>
       <c r="R21" s="7" t="str">
         <f t="shared" si="10"/>
-        <v>食べた</v>
+        <v>食べたい</v>
       </c>
       <c r="S21" s="7" t="str">
         <f t="shared" si="11"/>
+        <v>たべたい</v>
+      </c>
+      <c r="T21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="U21" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>たべ</v>
+      </c>
+      <c r="V21" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>食べない</v>
+      </c>
+      <c r="W21" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>たべない</v>
+      </c>
+      <c r="X21" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>食べなかった</v>
+      </c>
+      <c r="Y21" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>たべなかった</v>
+      </c>
+      <c r="Z21" s="7" t="str">
+        <f t="shared" si="20"/>
+        <v>食べた</v>
+      </c>
+      <c r="AA21" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB21" s="7" t="str">
+        <f t="shared" si="21"/>
         <v>食べて</v>
       </c>
+      <c r="AC21" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>たべて</v>
+      </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A22" s="7" t="s">
         <v>131</v>
       </c>
@@ -2547,41 +3500,80 @@
       </c>
       <c r="K22" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>寝ました</v>
+        <v>ねません</v>
       </c>
       <c r="L22" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>寝ませんでした</v>
+        <v>寝ました</v>
       </c>
       <c r="M22" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>寝ましょう</v>
+        <v>ねました</v>
       </c>
       <c r="N22" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>寝たい</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>133</v>
+        <v>寝ませんでした</v>
+      </c>
+      <c r="O22" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>ねませんでした</v>
       </c>
       <c r="P22" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>寝ない</v>
+        <f t="shared" si="8"/>
+        <v>寝ましょう</v>
       </c>
       <c r="Q22" s="7" t="str">
         <f t="shared" si="9"/>
-        <v>寝なかった</v>
+        <v>ねましょう</v>
       </c>
       <c r="R22" s="7" t="str">
         <f t="shared" si="10"/>
-        <v>寝た</v>
+        <v>寝たい</v>
       </c>
       <c r="S22" s="7" t="str">
         <f t="shared" si="11"/>
+        <v>ねたい</v>
+      </c>
+      <c r="T22" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="U22" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>ね</v>
+      </c>
+      <c r="V22" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>寝ない</v>
+      </c>
+      <c r="W22" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>ねない</v>
+      </c>
+      <c r="X22" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>寝なかった</v>
+      </c>
+      <c r="Y22" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>ねなかった</v>
+      </c>
+      <c r="Z22" s="7" t="str">
+        <f t="shared" si="20"/>
+        <v>寝た</v>
+      </c>
+      <c r="AA22" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB22" s="7" t="str">
+        <f t="shared" si="21"/>
         <v>寝て</v>
       </c>
+      <c r="AC22" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>ねて</v>
+      </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A23" s="7" t="s">
         <v>134</v>
       </c>
@@ -2617,41 +3609,80 @@
       </c>
       <c r="K23" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>見ました</v>
+        <v>みません</v>
       </c>
       <c r="L23" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>見ませんでした</v>
+        <v>見ました</v>
       </c>
       <c r="M23" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>見ましょう</v>
+        <v>みました</v>
       </c>
       <c r="N23" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>見たい</v>
-      </c>
-      <c r="O23" s="7" t="s">
-        <v>136</v>
+        <v>見ませんでした</v>
+      </c>
+      <c r="O23" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>みませんでした</v>
       </c>
       <c r="P23" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>見ない</v>
+        <f t="shared" si="8"/>
+        <v>見ましょう</v>
       </c>
       <c r="Q23" s="7" t="str">
         <f t="shared" si="9"/>
-        <v>見なかった</v>
+        <v>みましょう</v>
       </c>
       <c r="R23" s="7" t="str">
         <f t="shared" si="10"/>
-        <v>見た</v>
+        <v>見たい</v>
       </c>
       <c r="S23" s="7" t="str">
         <f t="shared" si="11"/>
+        <v>みたい</v>
+      </c>
+      <c r="T23" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="U23" s="7" t="str">
+        <f t="shared" si="19"/>
+        <v>み</v>
+      </c>
+      <c r="V23" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>見ない</v>
+      </c>
+      <c r="W23" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>みない</v>
+      </c>
+      <c r="X23" s="7" t="str">
+        <f t="shared" si="17"/>
+        <v>見なかった</v>
+      </c>
+      <c r="Y23" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>みなかった</v>
+      </c>
+      <c r="Z23" s="7" t="str">
+        <f t="shared" si="20"/>
+        <v>見た</v>
+      </c>
+      <c r="AA23" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="AB23" s="7" t="str">
+        <f t="shared" si="21"/>
         <v>見て</v>
       </c>
+      <c r="AC23" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>みて</v>
+      </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A24" s="7" t="s">
         <v>137</v>
       </c>
@@ -2687,39 +3718,76 @@
       </c>
       <c r="K24" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>来ました</v>
+        <v>きません</v>
       </c>
       <c r="L24" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>来ませんでした</v>
+        <v>来ました</v>
       </c>
       <c r="M24" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>来ましょう</v>
+        <v>きました</v>
       </c>
       <c r="N24" s="7" t="str">
         <f t="shared" si="6"/>
-        <v>来たい</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>140</v>
+        <v>来ませんでした</v>
+      </c>
+      <c r="O24" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>きませんでした</v>
       </c>
       <c r="P24" s="7" t="str">
-        <f t="shared" si="7"/>
-        <v>来ない</v>
+        <f t="shared" si="8"/>
+        <v>来ましょう</v>
       </c>
       <c r="Q24" s="7" t="str">
         <f t="shared" si="9"/>
+        <v>きましょう</v>
+      </c>
+      <c r="R24" s="7" t="str">
+        <f t="shared" si="10"/>
+        <v>来たい</v>
+      </c>
+      <c r="S24" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>きたい</v>
+      </c>
+      <c r="T24" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="U24" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="V24" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>来ない</v>
+      </c>
+      <c r="W24" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>こない</v>
+      </c>
+      <c r="X24" s="7" t="str">
+        <f t="shared" si="17"/>
         <v>来なかった</v>
       </c>
-      <c r="R24" s="7" t="s">
+      <c r="Y24" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>こなかった</v>
+      </c>
+      <c r="Z24" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="S24" s="7" t="s">
+      <c r="AA24" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="AB24" s="7" t="s">
         <v>142</v>
       </c>
+      <c r="AC24" s="7" t="s">
+        <v>216</v>
+      </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.6">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.6">
       <c r="A25" s="7" t="s">
         <v>143</v>
       </c>
@@ -2755,35 +3823,72 @@
       </c>
       <c r="K25" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>しました</v>
+        <v>しません</v>
       </c>
       <c r="L25" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>しませんでした</v>
+        <v>しました</v>
       </c>
       <c r="M25" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>しましょう</v>
+        <v>しました</v>
       </c>
       <c r="N25" s="7" t="str">
         <f t="shared" si="6"/>
+        <v>しませんでした</v>
+      </c>
+      <c r="O25" s="7" t="str">
+        <f t="shared" si="7"/>
+        <v>しませんでした</v>
+      </c>
+      <c r="P25" s="7" t="str">
+        <f t="shared" si="8"/>
+        <v>しましょう</v>
+      </c>
+      <c r="Q25" s="7" t="str">
+        <f t="shared" si="9"/>
+        <v>しましょう</v>
+      </c>
+      <c r="R25" s="7" t="str">
+        <f t="shared" si="10"/>
         <v>したい</v>
       </c>
-      <c r="O25" s="7" t="s">
+      <c r="S25" s="7" t="str">
+        <f t="shared" si="11"/>
+        <v>したい</v>
+      </c>
+      <c r="T25" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="P25" s="7" t="str">
-        <f t="shared" si="7"/>
+      <c r="U25" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="V25" s="7" t="str">
+        <f t="shared" si="12"/>
         <v>しない</v>
       </c>
-      <c r="Q25" s="7" t="str">
-        <f>_xlfn.CONCAT(O25,"なかった")</f>
+      <c r="W25" s="7" t="str">
+        <f t="shared" si="12"/>
+        <v>しない</v>
+      </c>
+      <c r="X25" s="7" t="str">
+        <f>_xlfn.CONCAT(T25,"なかった")</f>
         <v>しなかった</v>
       </c>
-      <c r="R25" s="7" t="s">
+      <c r="Y25" s="7" t="str">
+        <f t="shared" si="18"/>
+        <v>しなかった</v>
+      </c>
+      <c r="Z25" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="S25" s="7" t="s">
+      <c r="AA25" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="AB25" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="AC25" s="7" t="s">
         <v>147</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed a few errors in the verbs.xlsx
</commit_message>
<xml_diff>
--- a/verbs.xlsx
+++ b/verbs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BradHunt\Documents\japanese-practice\verbs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4805F6E8-B036-41CB-8C7D-2EF7B1677EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADF9E73-283B-47DC-B42D-3CD0E1C7B218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1845" windowWidth="29040" windowHeight="15720" xr2:uid="{9921D540-D520-4E46-B0DA-C77DD5C34F2D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{9921D540-D520-4E46-B0DA-C77DD5C34F2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="244">
   <si>
     <t>Dictionary</t>
   </si>
@@ -753,13 +753,28 @@
   </si>
   <si>
     <t>いって</t>
+  </si>
+  <si>
+    <t>きか</t>
+  </si>
+  <si>
+    <t>のんで</t>
+  </si>
+  <si>
+    <t>よんで</t>
+  </si>
+  <si>
+    <t>およいで</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -777,6 +792,32 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Meiryo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Meiryo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Meiryo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Meiryo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Meiryo"/>
       <family val="2"/>
     </font>
@@ -859,7 +900,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -879,6 +920,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1213,38 +1260,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{566C2546-B21A-4059-8C0C-B1CB9D497EEB}">
-  <dimension ref="A1:AH25"/>
+  <dimension ref="A1:AH28"/>
   <sheetFormatPr defaultRowHeight="17.5" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="12.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.08984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.08984375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="42.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.08984375" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="39.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.1796875" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="38.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="36.08984375" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="30.08984375" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17" style="6" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="29.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="39" style="6" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="25.6328125" style="6" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="35.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="28.1796875" style="6" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="38" style="6" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9.36328125" style="6" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.6328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="38.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.6328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="29" style="6" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="38.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="25.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="34.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="27.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="37.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9" style="6" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.36328125" style="6" bestFit="1" customWidth="1"/>
     <col min="30" max="34" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
@@ -1338,16 +1385,16 @@
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>149</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="6" t="s">
@@ -1363,7 +1410,7 @@
         <f>_xlfn.CONCAT(F2,"ます")</f>
         <v>行きます</v>
       </c>
-      <c r="I2" s="7" t="str">
+      <c r="I2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"ます")</f>
         <v>いきます</v>
       </c>
@@ -1371,7 +1418,7 @@
         <f>_xlfn.CONCAT(F2,"ません")</f>
         <v>行きません</v>
       </c>
-      <c r="K2" s="7" t="str">
+      <c r="K2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"ません")</f>
         <v>いきません</v>
       </c>
@@ -1379,7 +1426,7 @@
         <f>_xlfn.CONCAT(F2,"ました")</f>
         <v>行きました</v>
       </c>
-      <c r="M2" s="7" t="str">
+      <c r="M2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"ました")</f>
         <v>いきました</v>
       </c>
@@ -1387,7 +1434,7 @@
         <f>_xlfn.CONCAT(F2,"ませんでした")</f>
         <v>行きませんでした</v>
       </c>
-      <c r="O2" s="7" t="str">
+      <c r="O2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"ませんでした")</f>
         <v>いきませんでした</v>
       </c>
@@ -1395,7 +1442,7 @@
         <f>_xlfn.CONCAT(F2,"ましょう")</f>
         <v>行きましょう</v>
       </c>
-      <c r="Q2" s="7" t="str">
+      <c r="Q2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"ましょう")</f>
         <v>いきましょう</v>
       </c>
@@ -1403,7 +1450,7 @@
         <f>_xlfn.CONCAT(F2,"たい")</f>
         <v>行きたい</v>
       </c>
-      <c r="S2" s="7" t="str">
+      <c r="S2" s="9" t="str">
         <f>_xlfn.CONCAT(G2,"たい")</f>
         <v>いきたい</v>
       </c>
@@ -1417,7 +1464,7 @@
         <f>_xlfn.CONCAT(T2,"ない")</f>
         <v>行かない</v>
       </c>
-      <c r="W2" s="7" t="str">
+      <c r="W2" s="9" t="str">
         <f>_xlfn.CONCAT(U2,"ない")</f>
         <v>いかない</v>
       </c>
@@ -1425,34 +1472,34 @@
         <f>_xlfn.CONCAT(T2,"なかった")</f>
         <v>行かなかった</v>
       </c>
-      <c r="Y2" s="7" t="str">
+      <c r="Y2" s="9" t="str">
         <f>_xlfn.CONCAT(U2,"なかった")</f>
         <v>いかなかった</v>
       </c>
       <c r="Z2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="AA2" s="8" t="s">
+      <c r="AA2" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="AB2" s="8" t="s">
+      <c r="AB2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="AC2" s="8" t="s">
+      <c r="AC2" s="10" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="9" t="s">
         <v>150</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
@@ -1468,7 +1515,7 @@
         <f t="shared" ref="H3:H25" si="0">_xlfn.CONCAT(F3,"ます")</f>
         <v>帰ります</v>
       </c>
-      <c r="I3" s="7" t="str">
+      <c r="I3" s="9" t="str">
         <f t="shared" ref="I3:I25" si="1">_xlfn.CONCAT(G3,"ます")</f>
         <v>かえります</v>
       </c>
@@ -1476,7 +1523,7 @@
         <f t="shared" ref="J3:J25" si="2">_xlfn.CONCAT(F3,"ません")</f>
         <v>帰りません</v>
       </c>
-      <c r="K3" s="7" t="str">
+      <c r="K3" s="9" t="str">
         <f t="shared" ref="K3:K25" si="3">_xlfn.CONCAT(G3,"ません")</f>
         <v>かえりません</v>
       </c>
@@ -1484,7 +1531,7 @@
         <f t="shared" ref="L3:L25" si="4">_xlfn.CONCAT(F3,"ました")</f>
         <v>帰りました</v>
       </c>
-      <c r="M3" s="7" t="str">
+      <c r="M3" s="9" t="str">
         <f t="shared" ref="M3:M25" si="5">_xlfn.CONCAT(G3,"ました")</f>
         <v>かえりました</v>
       </c>
@@ -1492,7 +1539,7 @@
         <f t="shared" ref="N3:N25" si="6">_xlfn.CONCAT(F3,"ませんでした")</f>
         <v>帰りませんでした</v>
       </c>
-      <c r="O3" s="7" t="str">
+      <c r="O3" s="9" t="str">
         <f t="shared" ref="O3:O25" si="7">_xlfn.CONCAT(G3,"ませんでした")</f>
         <v>かえりませんでした</v>
       </c>
@@ -1500,7 +1547,7 @@
         <f t="shared" ref="P3:P25" si="8">_xlfn.CONCAT(F3,"ましょう")</f>
         <v>帰りましょう</v>
       </c>
-      <c r="Q3" s="7" t="str">
+      <c r="Q3" s="9" t="str">
         <f t="shared" ref="Q3:Q25" si="9">_xlfn.CONCAT(G3,"ましょう")</f>
         <v>かえりましょう</v>
       </c>
@@ -1508,7 +1555,7 @@
         <f t="shared" ref="R3:R25" si="10">_xlfn.CONCAT(F3,"たい")</f>
         <v>帰りたい</v>
       </c>
-      <c r="S3" s="7" t="str">
+      <c r="S3" s="9" t="str">
         <f t="shared" ref="S3:S25" si="11">_xlfn.CONCAT(G3,"たい")</f>
         <v>かえりたい</v>
       </c>
@@ -1522,7 +1569,7 @@
         <f t="shared" ref="V3:W25" si="12">_xlfn.CONCAT(T3,"ない")</f>
         <v>帰らない</v>
       </c>
-      <c r="W3" s="7" t="str">
+      <c r="W3" s="9" t="str">
         <f t="shared" ref="W3:W8" si="13">_xlfn.CONCAT(U3,"ない")</f>
         <v>かえらない</v>
       </c>
@@ -1530,35 +1577,35 @@
         <f t="shared" ref="X3:X8" si="14">_xlfn.CONCAT(T3,"なかった")</f>
         <v>帰らなかった</v>
       </c>
-      <c r="Y3" s="7" t="str">
+      <c r="Y3" s="9" t="str">
         <f t="shared" ref="Y3:Y8" si="15">_xlfn.CONCAT(U3,"なかった")</f>
         <v>かえらなかった</v>
       </c>
       <c r="Z3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="7" t="s">
+      <c r="AA3" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="AB3" s="7" t="s">
+      <c r="AB3" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="AC3" s="7" t="str">
+      <c r="AC3" s="9" t="str">
         <f>LEFT(AA3,LEN(AA3)-1) &amp; "て"</f>
         <v>かえって</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="9" t="s">
         <v>151</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="6" t="s">
@@ -1574,7 +1621,7 @@
         <f t="shared" si="0"/>
         <v>聞きます</v>
       </c>
-      <c r="I4" s="7" t="str">
+      <c r="I4" s="9" t="str">
         <f t="shared" si="1"/>
         <v>ききます</v>
       </c>
@@ -1582,7 +1629,7 @@
         <f t="shared" si="2"/>
         <v>聞きません</v>
       </c>
-      <c r="K4" s="7" t="str">
+      <c r="K4" s="9" t="str">
         <f t="shared" si="3"/>
         <v>ききません</v>
       </c>
@@ -1590,7 +1637,7 @@
         <f t="shared" si="4"/>
         <v>聞きました</v>
       </c>
-      <c r="M4" s="7" t="str">
+      <c r="M4" s="9" t="str">
         <f t="shared" si="5"/>
         <v>ききました</v>
       </c>
@@ -1598,7 +1645,7 @@
         <f t="shared" si="6"/>
         <v>聞きませんでした</v>
       </c>
-      <c r="O4" s="7" t="str">
+      <c r="O4" s="9" t="str">
         <f t="shared" si="7"/>
         <v>ききませんでした</v>
       </c>
@@ -1606,7 +1653,7 @@
         <f t="shared" si="8"/>
         <v>聞きましょう</v>
       </c>
-      <c r="Q4" s="7" t="str">
+      <c r="Q4" s="9" t="str">
         <f t="shared" si="9"/>
         <v>ききましょう</v>
       </c>
@@ -1614,7 +1661,7 @@
         <f t="shared" si="10"/>
         <v>聞きたい</v>
       </c>
-      <c r="S4" s="7" t="str">
+      <c r="S4" s="9" t="str">
         <f t="shared" si="11"/>
         <v>ききたい</v>
       </c>
@@ -1622,49 +1669,49 @@
         <v>34</v>
       </c>
       <c r="U4" s="7" t="s">
-        <v>206</v>
+        <v>239</v>
       </c>
       <c r="V4" s="7" t="str">
         <f t="shared" si="12"/>
         <v>聞かない</v>
       </c>
-      <c r="W4" s="7" t="str">
+      <c r="W4" s="9" t="str">
         <f t="shared" si="13"/>
-        <v>かかない</v>
+        <v>きかない</v>
       </c>
       <c r="X4" s="7" t="str">
         <f t="shared" si="14"/>
         <v>聞かなかった</v>
       </c>
-      <c r="Y4" s="7" t="str">
+      <c r="Y4" s="9" t="str">
         <f t="shared" si="15"/>
-        <v>かかなかった</v>
+        <v>きかなかった</v>
       </c>
       <c r="Z4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="AA4" s="7" t="s">
+      <c r="AA4" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="AB4" s="7" t="s">
+      <c r="AB4" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="AC4" s="7" t="str">
+      <c r="AC4" s="9" t="str">
         <f t="shared" ref="AC4:AC23" si="16">LEFT(AA4,LEN(AA4)-1) &amp; "て"</f>
         <v>きいて</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="9" t="s">
         <v>152</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="6" t="s">
@@ -1680,7 +1727,7 @@
         <f t="shared" si="0"/>
         <v>飲みます</v>
       </c>
-      <c r="I5" s="7" t="str">
+      <c r="I5" s="9" t="str">
         <f t="shared" si="1"/>
         <v>のみます</v>
       </c>
@@ -1688,7 +1735,7 @@
         <f t="shared" si="2"/>
         <v>飲みません</v>
       </c>
-      <c r="K5" s="7" t="str">
+      <c r="K5" s="9" t="str">
         <f t="shared" si="3"/>
         <v>のみません</v>
       </c>
@@ -1696,7 +1743,7 @@
         <f t="shared" si="4"/>
         <v>飲みました</v>
       </c>
-      <c r="M5" s="7" t="str">
+      <c r="M5" s="9" t="str">
         <f t="shared" si="5"/>
         <v>のみました</v>
       </c>
@@ -1704,7 +1751,7 @@
         <f t="shared" si="6"/>
         <v>飲みませんでした</v>
       </c>
-      <c r="O5" s="7" t="str">
+      <c r="O5" s="9" t="str">
         <f t="shared" si="7"/>
         <v>のみませんでした</v>
       </c>
@@ -1712,7 +1759,7 @@
         <f t="shared" si="8"/>
         <v>飲みましょう</v>
       </c>
-      <c r="Q5" s="7" t="str">
+      <c r="Q5" s="9" t="str">
         <f t="shared" si="9"/>
         <v>のみましょう</v>
       </c>
@@ -1720,7 +1767,7 @@
         <f t="shared" si="10"/>
         <v>飲みたい</v>
       </c>
-      <c r="S5" s="7" t="str">
+      <c r="S5" s="9" t="str">
         <f t="shared" si="11"/>
         <v>のみたい</v>
       </c>
@@ -1734,7 +1781,7 @@
         <f t="shared" si="12"/>
         <v>飲まない</v>
       </c>
-      <c r="W5" s="7" t="str">
+      <c r="W5" s="9" t="str">
         <f t="shared" si="13"/>
         <v>のまない</v>
       </c>
@@ -1742,35 +1789,34 @@
         <f t="shared" si="14"/>
         <v>飲まなかった</v>
       </c>
-      <c r="Y5" s="7" t="str">
+      <c r="Y5" s="9" t="str">
         <f t="shared" si="15"/>
         <v>のまなかった</v>
       </c>
       <c r="Z5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AA5" s="7" t="s">
+      <c r="AA5" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="AB5" s="7" t="s">
+      <c r="AB5" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="AC5" s="7" t="str">
-        <f t="shared" si="16"/>
-        <v>のんて</v>
+      <c r="AC5" s="9" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="9" t="s">
         <v>153</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E6" s="6" t="s">
@@ -1786,7 +1832,7 @@
         <f t="shared" si="0"/>
         <v>話します</v>
       </c>
-      <c r="I6" s="7" t="str">
+      <c r="I6" s="9" t="str">
         <f t="shared" si="1"/>
         <v>はなします</v>
       </c>
@@ -1794,7 +1840,7 @@
         <f t="shared" si="2"/>
         <v>話しません</v>
       </c>
-      <c r="K6" s="7" t="str">
+      <c r="K6" s="9" t="str">
         <f t="shared" si="3"/>
         <v>はなしません</v>
       </c>
@@ -1802,7 +1848,7 @@
         <f t="shared" si="4"/>
         <v>話しました</v>
       </c>
-      <c r="M6" s="7" t="str">
+      <c r="M6" s="9" t="str">
         <f t="shared" si="5"/>
         <v>はなしました</v>
       </c>
@@ -1810,7 +1856,7 @@
         <f t="shared" si="6"/>
         <v>話しませんでした</v>
       </c>
-      <c r="O6" s="7" t="str">
+      <c r="O6" s="9" t="str">
         <f t="shared" si="7"/>
         <v>はなしませんでした</v>
       </c>
@@ -1818,7 +1864,7 @@
         <f t="shared" si="8"/>
         <v>話しましょう</v>
       </c>
-      <c r="Q6" s="7" t="str">
+      <c r="Q6" s="9" t="str">
         <f t="shared" si="9"/>
         <v>はなしましょう</v>
       </c>
@@ -1826,7 +1872,7 @@
         <f t="shared" si="10"/>
         <v>話したい</v>
       </c>
-      <c r="S6" s="7" t="str">
+      <c r="S6" s="9" t="str">
         <f t="shared" si="11"/>
         <v>はなしたい</v>
       </c>
@@ -1840,7 +1886,7 @@
         <f t="shared" si="12"/>
         <v>話さない</v>
       </c>
-      <c r="W6" s="7" t="str">
+      <c r="W6" s="9" t="str">
         <f t="shared" si="13"/>
         <v>はなさない</v>
       </c>
@@ -1848,35 +1894,35 @@
         <f t="shared" si="14"/>
         <v>話さなかった</v>
       </c>
-      <c r="Y6" s="7" t="str">
+      <c r="Y6" s="9" t="str">
         <f t="shared" si="15"/>
         <v>はなさなかった</v>
       </c>
       <c r="Z6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AA6" s="7" t="s">
+      <c r="AA6" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="AB6" s="7" t="s">
+      <c r="AB6" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="AC6" s="7" t="str">
+      <c r="AC6" s="9" t="str">
         <f t="shared" si="16"/>
         <v>はなして</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="9" t="s">
         <v>154</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -1892,7 +1938,7 @@
         <f t="shared" si="0"/>
         <v>読みます</v>
       </c>
-      <c r="I7" s="7" t="str">
+      <c r="I7" s="9" t="str">
         <f t="shared" si="1"/>
         <v>よみます</v>
       </c>
@@ -1900,7 +1946,7 @@
         <f t="shared" si="2"/>
         <v>読みません</v>
       </c>
-      <c r="K7" s="7" t="str">
+      <c r="K7" s="9" t="str">
         <f t="shared" si="3"/>
         <v>よみません</v>
       </c>
@@ -1908,7 +1954,7 @@
         <f t="shared" si="4"/>
         <v>読みました</v>
       </c>
-      <c r="M7" s="7" t="str">
+      <c r="M7" s="9" t="str">
         <f t="shared" si="5"/>
         <v>よみました</v>
       </c>
@@ -1916,7 +1962,7 @@
         <f t="shared" si="6"/>
         <v>読みませんでした</v>
       </c>
-      <c r="O7" s="7" t="str">
+      <c r="O7" s="9" t="str">
         <f t="shared" si="7"/>
         <v>よみませんでした</v>
       </c>
@@ -1924,7 +1970,7 @@
         <f t="shared" si="8"/>
         <v>読みましょう</v>
       </c>
-      <c r="Q7" s="7" t="str">
+      <c r="Q7" s="9" t="str">
         <f t="shared" si="9"/>
         <v>よみましょう</v>
       </c>
@@ -1932,7 +1978,7 @@
         <f t="shared" si="10"/>
         <v>読みたい</v>
       </c>
-      <c r="S7" s="7" t="str">
+      <c r="S7" s="9" t="str">
         <f t="shared" si="11"/>
         <v>よみたい</v>
       </c>
@@ -1946,7 +1992,7 @@
         <f t="shared" si="12"/>
         <v>読まない</v>
       </c>
-      <c r="W7" s="7" t="str">
+      <c r="W7" s="9" t="str">
         <f t="shared" si="13"/>
         <v>よまない</v>
       </c>
@@ -1954,35 +2000,34 @@
         <f t="shared" si="14"/>
         <v>読まなかった</v>
       </c>
-      <c r="Y7" s="7" t="str">
+      <c r="Y7" s="9" t="str">
         <f t="shared" si="15"/>
         <v>よまなかった</v>
       </c>
       <c r="Z7" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="AA7" s="7" t="s">
+      <c r="AA7" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="AB7" s="7" t="s">
+      <c r="AB7" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="AC7" s="7" t="str">
-        <f t="shared" si="16"/>
-        <v>よんて</v>
+      <c r="AC7" s="9" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="9" t="s">
         <v>155</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E8" s="6" t="s">
@@ -1998,7 +2043,7 @@
         <f t="shared" si="0"/>
         <v>会います</v>
       </c>
-      <c r="I8" s="7" t="str">
+      <c r="I8" s="9" t="str">
         <f t="shared" si="1"/>
         <v>あいます</v>
       </c>
@@ -2006,7 +2051,7 @@
         <f t="shared" si="2"/>
         <v>会いません</v>
       </c>
-      <c r="K8" s="7" t="str">
+      <c r="K8" s="9" t="str">
         <f t="shared" si="3"/>
         <v>あいません</v>
       </c>
@@ -2014,7 +2059,7 @@
         <f t="shared" si="4"/>
         <v>会いました</v>
       </c>
-      <c r="M8" s="7" t="str">
+      <c r="M8" s="9" t="str">
         <f t="shared" si="5"/>
         <v>あいました</v>
       </c>
@@ -2022,7 +2067,7 @@
         <f t="shared" si="6"/>
         <v>会いませんでした</v>
       </c>
-      <c r="O8" s="7" t="str">
+      <c r="O8" s="9" t="str">
         <f t="shared" si="7"/>
         <v>あいませんでした</v>
       </c>
@@ -2030,7 +2075,7 @@
         <f t="shared" si="8"/>
         <v>会いましょう</v>
       </c>
-      <c r="Q8" s="7" t="str">
+      <c r="Q8" s="9" t="str">
         <f t="shared" si="9"/>
         <v>あいましょう</v>
       </c>
@@ -2038,7 +2083,7 @@
         <f t="shared" si="10"/>
         <v>会いたい</v>
       </c>
-      <c r="S8" s="7" t="str">
+      <c r="S8" s="9" t="str">
         <f t="shared" si="11"/>
         <v>あいたい</v>
       </c>
@@ -2052,7 +2097,7 @@
         <f t="shared" si="12"/>
         <v>会わない</v>
       </c>
-      <c r="W8" s="7" t="str">
+      <c r="W8" s="9" t="str">
         <f t="shared" si="13"/>
         <v>あわない</v>
       </c>
@@ -2060,35 +2105,35 @@
         <f t="shared" si="14"/>
         <v>会わなかった</v>
       </c>
-      <c r="Y8" s="7" t="str">
+      <c r="Y8" s="9" t="str">
         <f t="shared" si="15"/>
         <v>あわなかった</v>
       </c>
       <c r="Z8" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="AA8" s="7" t="s">
+      <c r="AA8" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="AB8" s="7" t="s">
+      <c r="AB8" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="AC8" s="7" t="str">
+      <c r="AC8" s="9" t="str">
         <f t="shared" si="16"/>
         <v>あって</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="9" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E9" s="6" t="s">
@@ -2104,7 +2149,7 @@
         <f t="shared" si="0"/>
         <v>あります</v>
       </c>
-      <c r="I9" s="7" t="str">
+      <c r="I9" s="9" t="str">
         <f t="shared" si="1"/>
         <v>あります</v>
       </c>
@@ -2112,7 +2157,7 @@
         <f t="shared" si="2"/>
         <v>ありません</v>
       </c>
-      <c r="K9" s="7" t="str">
+      <c r="K9" s="9" t="str">
         <f t="shared" si="3"/>
         <v>ありません</v>
       </c>
@@ -2120,7 +2165,7 @@
         <f t="shared" si="4"/>
         <v>ありました</v>
       </c>
-      <c r="M9" s="7" t="str">
+      <c r="M9" s="9" t="str">
         <f t="shared" si="5"/>
         <v>ありました</v>
       </c>
@@ -2128,7 +2173,7 @@
         <f t="shared" si="6"/>
         <v>ありませんでした</v>
       </c>
-      <c r="O9" s="7" t="str">
+      <c r="O9" s="9" t="str">
         <f t="shared" si="7"/>
         <v>ありませんでした</v>
       </c>
@@ -2136,7 +2181,7 @@
         <f t="shared" si="8"/>
         <v>ありましょう</v>
       </c>
-      <c r="Q9" s="7" t="str">
+      <c r="Q9" s="12" t="str">
         <f t="shared" si="9"/>
         <v>ありましょう</v>
       </c>
@@ -2144,7 +2189,7 @@
         <f t="shared" si="10"/>
         <v>ありたい</v>
       </c>
-      <c r="S9" s="7" t="str">
+      <c r="S9" s="12" t="str">
         <f t="shared" si="11"/>
         <v>ありたい</v>
       </c>
@@ -2157,40 +2202,40 @@
       <c r="V9" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="W9" s="8" t="s">
+      <c r="W9" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="X9" s="8" t="s">
+      <c r="X9" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="Y9" s="8" t="s">
+      <c r="Y9" s="10" t="s">
         <v>235</v>
       </c>
       <c r="Z9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="AA9" s="7" t="s">
+      <c r="AA9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="AB9" s="7" t="s">
+      <c r="AB9" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="AC9" s="7" t="str">
+      <c r="AC9" s="9" t="str">
         <f t="shared" si="16"/>
         <v>あって</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="9" t="s">
         <v>156</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E10" s="6" t="s">
@@ -2206,7 +2251,7 @@
         <f t="shared" si="0"/>
         <v>買います</v>
       </c>
-      <c r="I10" s="7" t="str">
+      <c r="I10" s="9" t="str">
         <f t="shared" si="1"/>
         <v>かいます</v>
       </c>
@@ -2214,7 +2259,7 @@
         <f t="shared" si="2"/>
         <v>買いません</v>
       </c>
-      <c r="K10" s="7" t="str">
+      <c r="K10" s="9" t="str">
         <f t="shared" si="3"/>
         <v>かいません</v>
       </c>
@@ -2222,7 +2267,7 @@
         <f t="shared" si="4"/>
         <v>買いました</v>
       </c>
-      <c r="M10" s="7" t="str">
+      <c r="M10" s="9" t="str">
         <f t="shared" si="5"/>
         <v>かいました</v>
       </c>
@@ -2230,7 +2275,7 @@
         <f t="shared" si="6"/>
         <v>買いませんでした</v>
       </c>
-      <c r="O10" s="7" t="str">
+      <c r="O10" s="9" t="str">
         <f t="shared" si="7"/>
         <v>かいませんでした</v>
       </c>
@@ -2238,7 +2283,7 @@
         <f t="shared" si="8"/>
         <v>買いましょう</v>
       </c>
-      <c r="Q10" s="7" t="str">
+      <c r="Q10" s="9" t="str">
         <f t="shared" si="9"/>
         <v>かいましょう</v>
       </c>
@@ -2246,7 +2291,7 @@
         <f t="shared" si="10"/>
         <v>買いたい</v>
       </c>
-      <c r="S10" s="7" t="str">
+      <c r="S10" s="9" t="str">
         <f t="shared" si="11"/>
         <v>かいたい</v>
       </c>
@@ -2260,7 +2305,7 @@
         <f t="shared" si="12"/>
         <v>買わない</v>
       </c>
-      <c r="W10" s="7" t="str">
+      <c r="W10" s="9" t="str">
         <f t="shared" si="12"/>
         <v>かわない</v>
       </c>
@@ -2268,35 +2313,35 @@
         <f>_xlfn.CONCAT(T10,"なかった")</f>
         <v>買わなかった</v>
       </c>
-      <c r="Y10" s="7" t="str">
+      <c r="Y10" s="9" t="str">
         <f>_xlfn.CONCAT(U10,"なかった")</f>
         <v>かわなかった</v>
       </c>
       <c r="Z10" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="AA10" s="7" t="s">
+      <c r="AA10" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="AB10" s="7" t="s">
+      <c r="AB10" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="AC10" s="7" t="str">
+      <c r="AC10" s="9" t="str">
         <f t="shared" si="16"/>
         <v>かって</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="9" t="s">
         <v>157</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -2312,7 +2357,7 @@
         <f t="shared" si="0"/>
         <v>書きます</v>
       </c>
-      <c r="I11" s="7" t="str">
+      <c r="I11" s="9" t="str">
         <f t="shared" si="1"/>
         <v>かきます</v>
       </c>
@@ -2320,7 +2365,7 @@
         <f t="shared" si="2"/>
         <v>書きません</v>
       </c>
-      <c r="K11" s="7" t="str">
+      <c r="K11" s="9" t="str">
         <f t="shared" si="3"/>
         <v>かきません</v>
       </c>
@@ -2328,7 +2373,7 @@
         <f t="shared" si="4"/>
         <v>書きました</v>
       </c>
-      <c r="M11" s="7" t="str">
+      <c r="M11" s="9" t="str">
         <f t="shared" si="5"/>
         <v>かきました</v>
       </c>
@@ -2336,7 +2381,7 @@
         <f t="shared" si="6"/>
         <v>書きませんでした</v>
       </c>
-      <c r="O11" s="7" t="str">
+      <c r="O11" s="9" t="str">
         <f t="shared" si="7"/>
         <v>かきませんでした</v>
       </c>
@@ -2344,7 +2389,7 @@
         <f t="shared" si="8"/>
         <v>書きましょう</v>
       </c>
-      <c r="Q11" s="7" t="str">
+      <c r="Q11" s="9" t="str">
         <f t="shared" si="9"/>
         <v>かきましょう</v>
       </c>
@@ -2352,7 +2397,7 @@
         <f t="shared" si="10"/>
         <v>書きたい</v>
       </c>
-      <c r="S11" s="7" t="str">
+      <c r="S11" s="9" t="str">
         <f t="shared" si="11"/>
         <v>かきたい</v>
       </c>
@@ -2366,7 +2411,7 @@
         <f t="shared" si="12"/>
         <v>書かない</v>
       </c>
-      <c r="W11" s="7" t="str">
+      <c r="W11" s="9" t="str">
         <f t="shared" si="12"/>
         <v>かかない</v>
       </c>
@@ -2374,35 +2419,35 @@
         <f t="shared" ref="X11:X24" si="17">_xlfn.CONCAT(T11,"なかった")</f>
         <v>書かなかった</v>
       </c>
-      <c r="Y11" s="7" t="str">
+      <c r="Y11" s="9" t="str">
         <f t="shared" ref="Y11:Y25" si="18">_xlfn.CONCAT(U11,"なかった")</f>
         <v>かかなかった</v>
       </c>
       <c r="Z11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="AA11" s="7" t="s">
+      <c r="AA11" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="AB11" s="7" t="s">
+      <c r="AB11" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="AC11" s="7" t="str">
+      <c r="AC11" s="9" t="str">
         <f t="shared" si="16"/>
         <v>かいて</v>
       </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="9" t="s">
         <v>158</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E12" s="6" t="s">
@@ -2418,7 +2463,7 @@
         <f t="shared" si="0"/>
         <v>撮ります</v>
       </c>
-      <c r="I12" s="7" t="str">
+      <c r="I12" s="9" t="str">
         <f t="shared" si="1"/>
         <v>とります</v>
       </c>
@@ -2426,7 +2471,7 @@
         <f t="shared" si="2"/>
         <v>撮りません</v>
       </c>
-      <c r="K12" s="7" t="str">
+      <c r="K12" s="9" t="str">
         <f t="shared" si="3"/>
         <v>とりません</v>
       </c>
@@ -2434,7 +2479,7 @@
         <f t="shared" si="4"/>
         <v>撮りました</v>
       </c>
-      <c r="M12" s="7" t="str">
+      <c r="M12" s="9" t="str">
         <f t="shared" si="5"/>
         <v>とりました</v>
       </c>
@@ -2442,7 +2487,7 @@
         <f t="shared" si="6"/>
         <v>撮りませんでした</v>
       </c>
-      <c r="O12" s="7" t="str">
+      <c r="O12" s="9" t="str">
         <f t="shared" si="7"/>
         <v>とりませんでした</v>
       </c>
@@ -2450,7 +2495,7 @@
         <f t="shared" si="8"/>
         <v>撮りましょう</v>
       </c>
-      <c r="Q12" s="7" t="str">
+      <c r="Q12" s="9" t="str">
         <f t="shared" si="9"/>
         <v>とりましょう</v>
       </c>
@@ -2458,7 +2503,7 @@
         <f t="shared" si="10"/>
         <v>撮りたい</v>
       </c>
-      <c r="S12" s="7" t="str">
+      <c r="S12" s="9" t="str">
         <f t="shared" si="11"/>
         <v>とりたい</v>
       </c>
@@ -2472,7 +2517,7 @@
         <f t="shared" si="12"/>
         <v>撮らない</v>
       </c>
-      <c r="W12" s="7" t="str">
+      <c r="W12" s="9" t="str">
         <f t="shared" si="12"/>
         <v>とらない</v>
       </c>
@@ -2480,35 +2525,35 @@
         <f t="shared" si="17"/>
         <v>撮らなかった</v>
       </c>
-      <c r="Y12" s="7" t="str">
+      <c r="Y12" s="9" t="str">
         <f t="shared" si="18"/>
         <v>とらなかった</v>
       </c>
       <c r="Z12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="AA12" s="7" t="s">
+      <c r="AA12" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="AB12" s="7" t="s">
+      <c r="AB12" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="AC12" s="7" t="str">
+      <c r="AC12" s="9" t="str">
         <f t="shared" si="16"/>
         <v>とって</v>
       </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="9" t="s">
         <v>159</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E13" s="6" t="s">
@@ -2524,7 +2569,7 @@
         <f t="shared" si="0"/>
         <v>待ちます</v>
       </c>
-      <c r="I13" s="7" t="str">
+      <c r="I13" s="9" t="str">
         <f t="shared" si="1"/>
         <v>まちます</v>
       </c>
@@ -2532,7 +2577,7 @@
         <f t="shared" si="2"/>
         <v>待ちません</v>
       </c>
-      <c r="K13" s="7" t="str">
+      <c r="K13" s="9" t="str">
         <f t="shared" si="3"/>
         <v>まちません</v>
       </c>
@@ -2540,7 +2585,7 @@
         <f t="shared" si="4"/>
         <v>待ちました</v>
       </c>
-      <c r="M13" s="7" t="str">
+      <c r="M13" s="9" t="str">
         <f t="shared" si="5"/>
         <v>まちました</v>
       </c>
@@ -2548,7 +2593,7 @@
         <f t="shared" si="6"/>
         <v>待ちませんでした</v>
       </c>
-      <c r="O13" s="7" t="str">
+      <c r="O13" s="9" t="str">
         <f t="shared" si="7"/>
         <v>まちませんでした</v>
       </c>
@@ -2556,7 +2601,7 @@
         <f t="shared" si="8"/>
         <v>待ちましょう</v>
       </c>
-      <c r="Q13" s="7" t="str">
+      <c r="Q13" s="9" t="str">
         <f t="shared" si="9"/>
         <v>まちましょう</v>
       </c>
@@ -2564,7 +2609,7 @@
         <f t="shared" si="10"/>
         <v>待ちたい</v>
       </c>
-      <c r="S13" s="7" t="str">
+      <c r="S13" s="9" t="str">
         <f t="shared" si="11"/>
         <v>まちたい</v>
       </c>
@@ -2578,7 +2623,7 @@
         <f t="shared" si="12"/>
         <v>待たない</v>
       </c>
-      <c r="W13" s="7" t="str">
+      <c r="W13" s="9" t="str">
         <f t="shared" si="12"/>
         <v>またない</v>
       </c>
@@ -2586,35 +2631,35 @@
         <f t="shared" si="17"/>
         <v>待たなかった</v>
       </c>
-      <c r="Y13" s="7" t="str">
+      <c r="Y13" s="9" t="str">
         <f t="shared" si="18"/>
         <v>またなかった</v>
       </c>
       <c r="Z13" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="AA13" s="7" t="s">
+      <c r="AA13" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="AB13" s="7" t="s">
+      <c r="AB13" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="AC13" s="7" t="str">
+      <c r="AC13" s="9" t="str">
         <f t="shared" si="16"/>
         <v>まって</v>
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="9" t="s">
         <v>160</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -2630,7 +2675,7 @@
         <f t="shared" si="0"/>
         <v>分かります</v>
       </c>
-      <c r="I14" s="7" t="str">
+      <c r="I14" s="9" t="str">
         <f t="shared" si="1"/>
         <v>わかります</v>
       </c>
@@ -2638,7 +2683,7 @@
         <f t="shared" si="2"/>
         <v>分かりません</v>
       </c>
-      <c r="K14" s="7" t="str">
+      <c r="K14" s="9" t="str">
         <f t="shared" si="3"/>
         <v>わかりません</v>
       </c>
@@ -2646,7 +2691,7 @@
         <f t="shared" si="4"/>
         <v>分かりました</v>
       </c>
-      <c r="M14" s="7" t="str">
+      <c r="M14" s="9" t="str">
         <f t="shared" si="5"/>
         <v>わかりました</v>
       </c>
@@ -2654,7 +2699,7 @@
         <f t="shared" si="6"/>
         <v>分かりませんでした</v>
       </c>
-      <c r="O14" s="7" t="str">
+      <c r="O14" s="9" t="str">
         <f t="shared" si="7"/>
         <v>わかりませんでした</v>
       </c>
@@ -2662,7 +2707,7 @@
         <f t="shared" si="8"/>
         <v>分かりましょう</v>
       </c>
-      <c r="Q14" s="7" t="str">
+      <c r="Q14" s="9" t="str">
         <f t="shared" si="9"/>
         <v>わかりましょう</v>
       </c>
@@ -2670,7 +2715,7 @@
         <f t="shared" si="10"/>
         <v>分かりたい</v>
       </c>
-      <c r="S14" s="7" t="str">
+      <c r="S14" s="9" t="str">
         <f t="shared" si="11"/>
         <v>わかりたい</v>
       </c>
@@ -2684,7 +2729,7 @@
         <f t="shared" si="12"/>
         <v>分からない</v>
       </c>
-      <c r="W14" s="7" t="str">
+      <c r="W14" s="9" t="str">
         <f t="shared" si="12"/>
         <v>わからない</v>
       </c>
@@ -2692,35 +2737,35 @@
         <f t="shared" si="17"/>
         <v>分からなかった</v>
       </c>
-      <c r="Y14" s="7" t="str">
+      <c r="Y14" s="9" t="str">
         <f t="shared" si="18"/>
         <v>わからなかった</v>
       </c>
       <c r="Z14" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="AA14" s="7" t="s">
+      <c r="AA14" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="AB14" s="7" t="s">
+      <c r="AB14" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="AC14" s="7" t="str">
+      <c r="AC14" s="9" t="str">
         <f t="shared" si="16"/>
         <v>わかって</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="9" t="s">
         <v>161</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E15" s="6" t="s">
@@ -2736,7 +2781,7 @@
         <f t="shared" si="0"/>
         <v>泳ぎます</v>
       </c>
-      <c r="I15" s="7" t="str">
+      <c r="I15" s="9" t="str">
         <f t="shared" si="1"/>
         <v>およぎます</v>
       </c>
@@ -2744,7 +2789,7 @@
         <f t="shared" si="2"/>
         <v>泳ぎません</v>
       </c>
-      <c r="K15" s="7" t="str">
+      <c r="K15" s="9" t="str">
         <f t="shared" si="3"/>
         <v>およぎません</v>
       </c>
@@ -2752,7 +2797,7 @@
         <f t="shared" si="4"/>
         <v>泳ぎました</v>
       </c>
-      <c r="M15" s="7" t="str">
+      <c r="M15" s="9" t="str">
         <f t="shared" si="5"/>
         <v>およぎました</v>
       </c>
@@ -2760,7 +2805,7 @@
         <f t="shared" si="6"/>
         <v>泳ぎませんでした</v>
       </c>
-      <c r="O15" s="7" t="str">
+      <c r="O15" s="9" t="str">
         <f t="shared" si="7"/>
         <v>およぎませんでした</v>
       </c>
@@ -2768,7 +2813,7 @@
         <f t="shared" si="8"/>
         <v>泳ぎましょう</v>
       </c>
-      <c r="Q15" s="7" t="str">
+      <c r="Q15" s="9" t="str">
         <f t="shared" si="9"/>
         <v>およぎましょう</v>
       </c>
@@ -2776,7 +2821,7 @@
         <f t="shared" si="10"/>
         <v>泳ぎたい</v>
       </c>
-      <c r="S15" s="7" t="str">
+      <c r="S15" s="9" t="str">
         <f t="shared" si="11"/>
         <v>およぎたい</v>
       </c>
@@ -2790,7 +2835,7 @@
         <f t="shared" si="12"/>
         <v>泳がない</v>
       </c>
-      <c r="W15" s="7" t="str">
+      <c r="W15" s="9" t="str">
         <f t="shared" si="12"/>
         <v>およがない</v>
       </c>
@@ -2798,35 +2843,34 @@
         <f t="shared" si="17"/>
         <v>泳がなかった</v>
       </c>
-      <c r="Y15" s="7" t="str">
+      <c r="Y15" s="9" t="str">
         <f t="shared" si="18"/>
         <v>およがなかった</v>
       </c>
       <c r="Z15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="AA15" s="7" t="s">
+      <c r="AA15" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="AB15" s="7" t="s">
+      <c r="AB15" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="AC15" s="7" t="str">
-        <f t="shared" si="16"/>
-        <v>およいて</v>
+      <c r="AC15" s="9" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="9" t="s">
         <v>162</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E16" s="6" t="s">
@@ -2842,7 +2886,7 @@
         <f t="shared" si="0"/>
         <v>乗ります</v>
       </c>
-      <c r="I16" s="7" t="str">
+      <c r="I16" s="9" t="str">
         <f t="shared" si="1"/>
         <v>のります</v>
       </c>
@@ -2850,7 +2894,7 @@
         <f t="shared" si="2"/>
         <v>乗りません</v>
       </c>
-      <c r="K16" s="7" t="str">
+      <c r="K16" s="9" t="str">
         <f t="shared" si="3"/>
         <v>のりません</v>
       </c>
@@ -2858,7 +2902,7 @@
         <f t="shared" si="4"/>
         <v>乗りました</v>
       </c>
-      <c r="M16" s="7" t="str">
+      <c r="M16" s="9" t="str">
         <f t="shared" si="5"/>
         <v>のりました</v>
       </c>
@@ -2866,7 +2910,7 @@
         <f t="shared" si="6"/>
         <v>乗りませんでした</v>
       </c>
-      <c r="O16" s="7" t="str">
+      <c r="O16" s="9" t="str">
         <f t="shared" si="7"/>
         <v>のりませんでした</v>
       </c>
@@ -2874,7 +2918,7 @@
         <f t="shared" si="8"/>
         <v>乗りましょう</v>
       </c>
-      <c r="Q16" s="7" t="str">
+      <c r="Q16" s="9" t="str">
         <f t="shared" si="9"/>
         <v>のりましょう</v>
       </c>
@@ -2882,7 +2926,7 @@
         <f t="shared" si="10"/>
         <v>乗りたい</v>
       </c>
-      <c r="S16" s="7" t="str">
+      <c r="S16" s="9" t="str">
         <f t="shared" si="11"/>
         <v>のりたい</v>
       </c>
@@ -2896,7 +2940,7 @@
         <f t="shared" si="12"/>
         <v>乗らない</v>
       </c>
-      <c r="W16" s="7" t="str">
+      <c r="W16" s="9" t="str">
         <f t="shared" si="12"/>
         <v>のらない</v>
       </c>
@@ -2904,35 +2948,35 @@
         <f t="shared" si="17"/>
         <v>乗らなかった</v>
       </c>
-      <c r="Y16" s="7" t="str">
+      <c r="Y16" s="9" t="str">
         <f t="shared" si="18"/>
         <v>のらなかった</v>
       </c>
       <c r="Z16" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="AA16" s="7" t="s">
+      <c r="AA16" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="AB16" s="7" t="s">
+      <c r="AB16" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="AC16" s="7" t="str">
+      <c r="AC16" s="9" t="str">
         <f t="shared" si="16"/>
         <v>のって</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="9" t="s">
         <v>111</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E17" s="6" t="s">
@@ -2948,7 +2992,7 @@
         <f t="shared" si="0"/>
         <v>やります</v>
       </c>
-      <c r="I17" s="7" t="str">
+      <c r="I17" s="9" t="str">
         <f t="shared" si="1"/>
         <v>やります</v>
       </c>
@@ -2956,7 +3000,7 @@
         <f t="shared" si="2"/>
         <v>やりません</v>
       </c>
-      <c r="K17" s="7" t="str">
+      <c r="K17" s="9" t="str">
         <f t="shared" si="3"/>
         <v>やりません</v>
       </c>
@@ -2964,7 +3008,7 @@
         <f t="shared" si="4"/>
         <v>やりました</v>
       </c>
-      <c r="M17" s="7" t="str">
+      <c r="M17" s="9" t="str">
         <f t="shared" si="5"/>
         <v>やりました</v>
       </c>
@@ -2972,7 +3016,7 @@
         <f t="shared" si="6"/>
         <v>やりませんでした</v>
       </c>
-      <c r="O17" s="7" t="str">
+      <c r="O17" s="9" t="str">
         <f t="shared" si="7"/>
         <v>やりませんでした</v>
       </c>
@@ -2980,7 +3024,7 @@
         <f t="shared" si="8"/>
         <v>やりましょう</v>
       </c>
-      <c r="Q17" s="7" t="str">
+      <c r="Q17" s="9" t="str">
         <f t="shared" si="9"/>
         <v>やりましょう</v>
       </c>
@@ -2988,7 +3032,7 @@
         <f t="shared" si="10"/>
         <v>やりたい</v>
       </c>
-      <c r="S17" s="7" t="str">
+      <c r="S17" s="9" t="str">
         <f t="shared" si="11"/>
         <v>やりたい</v>
       </c>
@@ -3002,7 +3046,7 @@
         <f t="shared" si="12"/>
         <v>やらない</v>
       </c>
-      <c r="W17" s="7" t="str">
+      <c r="W17" s="9" t="str">
         <f t="shared" si="12"/>
         <v>やらない</v>
       </c>
@@ -3010,35 +3054,35 @@
         <f t="shared" si="17"/>
         <v>やらなかった</v>
       </c>
-      <c r="Y17" s="7" t="str">
+      <c r="Y17" s="9" t="str">
         <f t="shared" si="18"/>
         <v>やらなかった</v>
       </c>
       <c r="Z17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="AA17" s="7" t="s">
+      <c r="AA17" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="AB17" s="7" t="s">
+      <c r="AB17" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="AC17" s="7" t="str">
+      <c r="AC17" s="9" t="str">
         <f t="shared" si="16"/>
         <v>やって</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="9" t="s">
         <v>163</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E18" s="6" t="s">
@@ -3054,7 +3098,7 @@
         <f t="shared" si="0"/>
         <v>出かけます</v>
       </c>
-      <c r="I18" s="7" t="str">
+      <c r="I18" s="9" t="str">
         <f t="shared" si="1"/>
         <v>でかけます</v>
       </c>
@@ -3062,7 +3106,7 @@
         <f t="shared" si="2"/>
         <v>出かけません</v>
       </c>
-      <c r="K18" s="7" t="str">
+      <c r="K18" s="9" t="str">
         <f t="shared" si="3"/>
         <v>でかけません</v>
       </c>
@@ -3070,7 +3114,7 @@
         <f t="shared" si="4"/>
         <v>出かけました</v>
       </c>
-      <c r="M18" s="7" t="str">
+      <c r="M18" s="9" t="str">
         <f t="shared" si="5"/>
         <v>でかけました</v>
       </c>
@@ -3078,7 +3122,7 @@
         <f t="shared" si="6"/>
         <v>出かけませんでした</v>
       </c>
-      <c r="O18" s="7" t="str">
+      <c r="O18" s="9" t="str">
         <f t="shared" si="7"/>
         <v>でかけませんでした</v>
       </c>
@@ -3086,7 +3130,7 @@
         <f t="shared" si="8"/>
         <v>出かけましょう</v>
       </c>
-      <c r="Q18" s="7" t="str">
+      <c r="Q18" s="9" t="str">
         <f t="shared" si="9"/>
         <v>でかけましょう</v>
       </c>
@@ -3094,7 +3138,7 @@
         <f t="shared" si="10"/>
         <v>出かけたい</v>
       </c>
-      <c r="S18" s="7" t="str">
+      <c r="S18" s="9" t="str">
         <f t="shared" si="11"/>
         <v>でかけたい</v>
       </c>
@@ -3109,7 +3153,7 @@
         <f t="shared" si="12"/>
         <v>出かけない</v>
       </c>
-      <c r="W18" s="7" t="str">
+      <c r="W18" s="9" t="str">
         <f t="shared" si="12"/>
         <v>でかけない</v>
       </c>
@@ -3117,7 +3161,7 @@
         <f t="shared" si="17"/>
         <v>出かけなかった</v>
       </c>
-      <c r="Y18" s="7" t="str">
+      <c r="Y18" s="9" t="str">
         <f t="shared" si="18"/>
         <v>でかけなかった</v>
       </c>
@@ -3125,29 +3169,29 @@
         <f>_xlfn.CONCAT(F18,"た")</f>
         <v>出かけた</v>
       </c>
-      <c r="AA18" s="7" t="s">
+      <c r="AA18" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="AB18" s="7" t="str">
+      <c r="AB18" s="14" t="str">
         <f>_xlfn.CONCAT(F18,"て")</f>
         <v>出かけて</v>
       </c>
-      <c r="AC18" s="7" t="str">
+      <c r="AC18" s="9" t="str">
         <f t="shared" si="16"/>
         <v>でかけて</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="9" t="s">
         <v>122</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E19" s="6" t="s">
@@ -3163,7 +3207,7 @@
         <f t="shared" si="0"/>
         <v>います</v>
       </c>
-      <c r="I19" s="7" t="str">
+      <c r="I19" s="9" t="str">
         <f t="shared" si="1"/>
         <v>います</v>
       </c>
@@ -3171,7 +3215,7 @@
         <f t="shared" si="2"/>
         <v>いません</v>
       </c>
-      <c r="K19" s="7" t="str">
+      <c r="K19" s="9" t="str">
         <f t="shared" si="3"/>
         <v>いません</v>
       </c>
@@ -3179,7 +3223,7 @@
         <f t="shared" si="4"/>
         <v>いました</v>
       </c>
-      <c r="M19" s="7" t="str">
+      <c r="M19" s="9" t="str">
         <f t="shared" si="5"/>
         <v>いました</v>
       </c>
@@ -3187,7 +3231,7 @@
         <f t="shared" si="6"/>
         <v>いませんでした</v>
       </c>
-      <c r="O19" s="7" t="str">
+      <c r="O19" s="9" t="str">
         <f t="shared" si="7"/>
         <v>いませんでした</v>
       </c>
@@ -3195,7 +3239,7 @@
         <f t="shared" si="8"/>
         <v>いましょう</v>
       </c>
-      <c r="Q19" s="7" t="str">
+      <c r="Q19" s="9" t="str">
         <f t="shared" si="9"/>
         <v>いましょう</v>
       </c>
@@ -3203,7 +3247,7 @@
         <f t="shared" si="10"/>
         <v>いたい</v>
       </c>
-      <c r="S19" s="7" t="str">
+      <c r="S19" s="9" t="str">
         <f t="shared" si="11"/>
         <v>いたい</v>
       </c>
@@ -3218,7 +3262,7 @@
         <f t="shared" si="12"/>
         <v>いない</v>
       </c>
-      <c r="W19" s="7" t="str">
+      <c r="W19" s="9" t="str">
         <f t="shared" si="12"/>
         <v>いない</v>
       </c>
@@ -3226,7 +3270,7 @@
         <f t="shared" si="17"/>
         <v>いなかった</v>
       </c>
-      <c r="Y19" s="7" t="str">
+      <c r="Y19" s="9" t="str">
         <f t="shared" si="18"/>
         <v>いなかった</v>
       </c>
@@ -3234,29 +3278,29 @@
         <f t="shared" ref="Z19:Z23" si="20">_xlfn.CONCAT(F19,"た")</f>
         <v>いた</v>
       </c>
-      <c r="AA19" s="7" t="s">
+      <c r="AA19" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="AB19" s="7" t="str">
+      <c r="AB19" s="14" t="str">
         <f t="shared" ref="AB19:AB23" si="21">_xlfn.CONCAT(F19,"て")</f>
         <v>いて</v>
       </c>
-      <c r="AC19" s="7" t="str">
+      <c r="AC19" s="9" t="str">
         <f t="shared" si="16"/>
         <v>いて</v>
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="9" t="s">
         <v>164</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E20" s="6" t="s">
@@ -3272,7 +3316,7 @@
         <f t="shared" si="0"/>
         <v>起きます</v>
       </c>
-      <c r="I20" s="7" t="str">
+      <c r="I20" s="9" t="str">
         <f t="shared" si="1"/>
         <v>おきます</v>
       </c>
@@ -3280,7 +3324,7 @@
         <f t="shared" si="2"/>
         <v>起きません</v>
       </c>
-      <c r="K20" s="7" t="str">
+      <c r="K20" s="9" t="str">
         <f t="shared" si="3"/>
         <v>おきません</v>
       </c>
@@ -3288,7 +3332,7 @@
         <f t="shared" si="4"/>
         <v>起きました</v>
       </c>
-      <c r="M20" s="7" t="str">
+      <c r="M20" s="9" t="str">
         <f t="shared" si="5"/>
         <v>おきました</v>
       </c>
@@ -3296,7 +3340,7 @@
         <f t="shared" si="6"/>
         <v>起きませんでした</v>
       </c>
-      <c r="O20" s="7" t="str">
+      <c r="O20" s="9" t="str">
         <f t="shared" si="7"/>
         <v>おきませんでした</v>
       </c>
@@ -3304,7 +3348,7 @@
         <f t="shared" si="8"/>
         <v>起きましょう</v>
       </c>
-      <c r="Q20" s="7" t="str">
+      <c r="Q20" s="9" t="str">
         <f t="shared" si="9"/>
         <v>おきましょう</v>
       </c>
@@ -3312,7 +3356,7 @@
         <f t="shared" si="10"/>
         <v>起きたい</v>
       </c>
-      <c r="S20" s="7" t="str">
+      <c r="S20" s="9" t="str">
         <f t="shared" si="11"/>
         <v>おきたい</v>
       </c>
@@ -3327,7 +3371,7 @@
         <f t="shared" si="12"/>
         <v>起きない</v>
       </c>
-      <c r="W20" s="7" t="str">
+      <c r="W20" s="9" t="str">
         <f t="shared" si="12"/>
         <v>おきない</v>
       </c>
@@ -3335,7 +3379,7 @@
         <f t="shared" si="17"/>
         <v>起きなかった</v>
       </c>
-      <c r="Y20" s="7" t="str">
+      <c r="Y20" s="9" t="str">
         <f t="shared" si="18"/>
         <v>おきなかった</v>
       </c>
@@ -3343,29 +3387,29 @@
         <f t="shared" si="20"/>
         <v>起きた</v>
       </c>
-      <c r="AA20" s="7" t="s">
+      <c r="AA20" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="AB20" s="7" t="str">
+      <c r="AB20" s="14" t="str">
         <f t="shared" si="21"/>
         <v>起きて</v>
       </c>
-      <c r="AC20" s="7" t="str">
+      <c r="AC20" s="9" t="str">
         <f t="shared" si="16"/>
         <v>おきて</v>
       </c>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="9" t="s">
         <v>165</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E21" s="6" t="s">
@@ -3381,7 +3425,7 @@
         <f t="shared" si="0"/>
         <v>食べます</v>
       </c>
-      <c r="I21" s="7" t="str">
+      <c r="I21" s="9" t="str">
         <f t="shared" si="1"/>
         <v>たべます</v>
       </c>
@@ -3389,7 +3433,7 @@
         <f t="shared" si="2"/>
         <v>食べません</v>
       </c>
-      <c r="K21" s="7" t="str">
+      <c r="K21" s="9" t="str">
         <f t="shared" si="3"/>
         <v>たべません</v>
       </c>
@@ -3397,7 +3441,7 @@
         <f t="shared" si="4"/>
         <v>食べました</v>
       </c>
-      <c r="M21" s="7" t="str">
+      <c r="M21" s="9" t="str">
         <f t="shared" si="5"/>
         <v>たべました</v>
       </c>
@@ -3405,7 +3449,7 @@
         <f t="shared" si="6"/>
         <v>食べませんでした</v>
       </c>
-      <c r="O21" s="7" t="str">
+      <c r="O21" s="9" t="str">
         <f t="shared" si="7"/>
         <v>たべませんでした</v>
       </c>
@@ -3413,7 +3457,7 @@
         <f t="shared" si="8"/>
         <v>食べましょう</v>
       </c>
-      <c r="Q21" s="7" t="str">
+      <c r="Q21" s="9" t="str">
         <f t="shared" si="9"/>
         <v>たべましょう</v>
       </c>
@@ -3421,7 +3465,7 @@
         <f t="shared" si="10"/>
         <v>食べたい</v>
       </c>
-      <c r="S21" s="7" t="str">
+      <c r="S21" s="9" t="str">
         <f t="shared" si="11"/>
         <v>たべたい</v>
       </c>
@@ -3436,7 +3480,7 @@
         <f t="shared" si="12"/>
         <v>食べない</v>
       </c>
-      <c r="W21" s="7" t="str">
+      <c r="W21" s="9" t="str">
         <f t="shared" si="12"/>
         <v>たべない</v>
       </c>
@@ -3444,7 +3488,7 @@
         <f t="shared" si="17"/>
         <v>食べなかった</v>
       </c>
-      <c r="Y21" s="7" t="str">
+      <c r="Y21" s="9" t="str">
         <f t="shared" si="18"/>
         <v>たべなかった</v>
       </c>
@@ -3452,29 +3496,29 @@
         <f t="shared" si="20"/>
         <v>食べた</v>
       </c>
-      <c r="AA21" s="7" t="s">
+      <c r="AA21" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AB21" s="7" t="str">
+      <c r="AB21" s="14" t="str">
         <f t="shared" si="21"/>
         <v>食べて</v>
       </c>
-      <c r="AC21" s="7" t="str">
+      <c r="AC21" s="9" t="str">
         <f t="shared" si="16"/>
         <v>たべて</v>
       </c>
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="9" t="s">
         <v>166</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E22" s="6" t="s">
@@ -3490,7 +3534,7 @@
         <f t="shared" si="0"/>
         <v>寝ます</v>
       </c>
-      <c r="I22" s="7" t="str">
+      <c r="I22" s="9" t="str">
         <f t="shared" si="1"/>
         <v>ねます</v>
       </c>
@@ -3498,7 +3542,7 @@
         <f t="shared" si="2"/>
         <v>寝ません</v>
       </c>
-      <c r="K22" s="7" t="str">
+      <c r="K22" s="9" t="str">
         <f t="shared" si="3"/>
         <v>ねません</v>
       </c>
@@ -3506,7 +3550,7 @@
         <f t="shared" si="4"/>
         <v>寝ました</v>
       </c>
-      <c r="M22" s="7" t="str">
+      <c r="M22" s="9" t="str">
         <f t="shared" si="5"/>
         <v>ねました</v>
       </c>
@@ -3514,7 +3558,7 @@
         <f t="shared" si="6"/>
         <v>寝ませんでした</v>
       </c>
-      <c r="O22" s="7" t="str">
+      <c r="O22" s="9" t="str">
         <f t="shared" si="7"/>
         <v>ねませんでした</v>
       </c>
@@ -3522,7 +3566,7 @@
         <f t="shared" si="8"/>
         <v>寝ましょう</v>
       </c>
-      <c r="Q22" s="7" t="str">
+      <c r="Q22" s="9" t="str">
         <f t="shared" si="9"/>
         <v>ねましょう</v>
       </c>
@@ -3530,7 +3574,7 @@
         <f t="shared" si="10"/>
         <v>寝たい</v>
       </c>
-      <c r="S22" s="7" t="str">
+      <c r="S22" s="9" t="str">
         <f t="shared" si="11"/>
         <v>ねたい</v>
       </c>
@@ -3545,7 +3589,7 @@
         <f t="shared" si="12"/>
         <v>寝ない</v>
       </c>
-      <c r="W22" s="7" t="str">
+      <c r="W22" s="9" t="str">
         <f t="shared" si="12"/>
         <v>ねない</v>
       </c>
@@ -3553,7 +3597,7 @@
         <f t="shared" si="17"/>
         <v>寝なかった</v>
       </c>
-      <c r="Y22" s="7" t="str">
+      <c r="Y22" s="9" t="str">
         <f t="shared" si="18"/>
         <v>ねなかった</v>
       </c>
@@ -3561,29 +3605,29 @@
         <f t="shared" si="20"/>
         <v>寝た</v>
       </c>
-      <c r="AA22" s="7" t="s">
+      <c r="AA22" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="AB22" s="7" t="str">
+      <c r="AB22" s="14" t="str">
         <f t="shared" si="21"/>
         <v>寝て</v>
       </c>
-      <c r="AC22" s="7" t="str">
+      <c r="AC22" s="9" t="str">
         <f t="shared" si="16"/>
         <v>ねて</v>
       </c>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="9" t="s">
         <v>167</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="11" t="s">
         <v>119</v>
       </c>
       <c r="E23" s="6" t="s">
@@ -3599,7 +3643,7 @@
         <f t="shared" si="0"/>
         <v>見ます</v>
       </c>
-      <c r="I23" s="7" t="str">
+      <c r="I23" s="9" t="str">
         <f t="shared" si="1"/>
         <v>みます</v>
       </c>
@@ -3607,7 +3651,7 @@
         <f t="shared" si="2"/>
         <v>見ません</v>
       </c>
-      <c r="K23" s="7" t="str">
+      <c r="K23" s="9" t="str">
         <f t="shared" si="3"/>
         <v>みません</v>
       </c>
@@ -3615,7 +3659,7 @@
         <f t="shared" si="4"/>
         <v>見ました</v>
       </c>
-      <c r="M23" s="7" t="str">
+      <c r="M23" s="9" t="str">
         <f t="shared" si="5"/>
         <v>みました</v>
       </c>
@@ -3623,7 +3667,7 @@
         <f t="shared" si="6"/>
         <v>見ませんでした</v>
       </c>
-      <c r="O23" s="7" t="str">
+      <c r="O23" s="9" t="str">
         <f t="shared" si="7"/>
         <v>みませんでした</v>
       </c>
@@ -3631,7 +3675,7 @@
         <f t="shared" si="8"/>
         <v>見ましょう</v>
       </c>
-      <c r="Q23" s="7" t="str">
+      <c r="Q23" s="9" t="str">
         <f t="shared" si="9"/>
         <v>みましょう</v>
       </c>
@@ -3639,7 +3683,7 @@
         <f t="shared" si="10"/>
         <v>見たい</v>
       </c>
-      <c r="S23" s="7" t="str">
+      <c r="S23" s="9" t="str">
         <f t="shared" si="11"/>
         <v>みたい</v>
       </c>
@@ -3654,7 +3698,7 @@
         <f t="shared" si="12"/>
         <v>見ない</v>
       </c>
-      <c r="W23" s="7" t="str">
+      <c r="W23" s="9" t="str">
         <f t="shared" si="12"/>
         <v>みない</v>
       </c>
@@ -3662,7 +3706,7 @@
         <f t="shared" si="17"/>
         <v>見なかった</v>
       </c>
-      <c r="Y23" s="7" t="str">
+      <c r="Y23" s="9" t="str">
         <f t="shared" si="18"/>
         <v>みなかった</v>
       </c>
@@ -3670,29 +3714,29 @@
         <f t="shared" si="20"/>
         <v>見た</v>
       </c>
-      <c r="AA23" s="7" t="s">
+      <c r="AA23" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="AB23" s="7" t="str">
+      <c r="AB23" s="14" t="str">
         <f t="shared" si="21"/>
         <v>見て</v>
       </c>
-      <c r="AC23" s="7" t="str">
+      <c r="AC23" s="9" t="str">
         <f t="shared" si="16"/>
         <v>みて</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="9" t="s">
         <v>168</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="11" t="s">
         <v>139</v>
       </c>
       <c r="E24" s="6" t="s">
@@ -3708,7 +3752,7 @@
         <f t="shared" si="0"/>
         <v>来ます</v>
       </c>
-      <c r="I24" s="7" t="str">
+      <c r="I24" s="9" t="str">
         <f t="shared" si="1"/>
         <v>きます</v>
       </c>
@@ -3716,7 +3760,7 @@
         <f t="shared" si="2"/>
         <v>来ません</v>
       </c>
-      <c r="K24" s="7" t="str">
+      <c r="K24" s="9" t="str">
         <f t="shared" si="3"/>
         <v>きません</v>
       </c>
@@ -3724,7 +3768,7 @@
         <f t="shared" si="4"/>
         <v>来ました</v>
       </c>
-      <c r="M24" s="7" t="str">
+      <c r="M24" s="9" t="str">
         <f t="shared" si="5"/>
         <v>きました</v>
       </c>
@@ -3732,7 +3776,7 @@
         <f t="shared" si="6"/>
         <v>来ませんでした</v>
       </c>
-      <c r="O24" s="7" t="str">
+      <c r="O24" s="9" t="str">
         <f t="shared" si="7"/>
         <v>きませんでした</v>
       </c>
@@ -3740,7 +3784,7 @@
         <f t="shared" si="8"/>
         <v>来ましょう</v>
       </c>
-      <c r="Q24" s="7" t="str">
+      <c r="Q24" s="9" t="str">
         <f t="shared" si="9"/>
         <v>きましょう</v>
       </c>
@@ -3748,7 +3792,7 @@
         <f t="shared" si="10"/>
         <v>来たい</v>
       </c>
-      <c r="S24" s="7" t="str">
+      <c r="S24" s="12" t="str">
         <f t="shared" si="11"/>
         <v>きたい</v>
       </c>
@@ -3762,7 +3806,7 @@
         <f t="shared" si="12"/>
         <v>来ない</v>
       </c>
-      <c r="W24" s="7" t="str">
+      <c r="W24" s="9" t="str">
         <f t="shared" si="12"/>
         <v>こない</v>
       </c>
@@ -3770,34 +3814,34 @@
         <f t="shared" si="17"/>
         <v>来なかった</v>
       </c>
-      <c r="Y24" s="7" t="str">
+      <c r="Y24" s="9" t="str">
         <f t="shared" si="18"/>
         <v>こなかった</v>
       </c>
       <c r="Z24" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="AA24" s="7" t="s">
+      <c r="AA24" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="AB24" s="7" t="s">
+      <c r="AB24" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="AC24" s="7" t="s">
+      <c r="AC24" s="9" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="9" t="s">
         <v>143</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="11" t="s">
         <v>139</v>
       </c>
       <c r="E25" s="6" t="s">
@@ -3813,7 +3857,7 @@
         <f t="shared" si="0"/>
         <v>します</v>
       </c>
-      <c r="I25" s="7" t="str">
+      <c r="I25" s="9" t="str">
         <f t="shared" si="1"/>
         <v>します</v>
       </c>
@@ -3821,7 +3865,7 @@
         <f t="shared" si="2"/>
         <v>しません</v>
       </c>
-      <c r="K25" s="7" t="str">
+      <c r="K25" s="9" t="str">
         <f t="shared" si="3"/>
         <v>しません</v>
       </c>
@@ -3829,7 +3873,7 @@
         <f t="shared" si="4"/>
         <v>しました</v>
       </c>
-      <c r="M25" s="7" t="str">
+      <c r="M25" s="9" t="str">
         <f t="shared" si="5"/>
         <v>しました</v>
       </c>
@@ -3837,7 +3881,7 @@
         <f t="shared" si="6"/>
         <v>しませんでした</v>
       </c>
-      <c r="O25" s="7" t="str">
+      <c r="O25" s="9" t="str">
         <f t="shared" si="7"/>
         <v>しませんでした</v>
       </c>
@@ -3845,7 +3889,7 @@
         <f t="shared" si="8"/>
         <v>しましょう</v>
       </c>
-      <c r="Q25" s="7" t="str">
+      <c r="Q25" s="9" t="str">
         <f t="shared" si="9"/>
         <v>しましょう</v>
       </c>
@@ -3853,7 +3897,7 @@
         <f t="shared" si="10"/>
         <v>したい</v>
       </c>
-      <c r="S25" s="7" t="str">
+      <c r="S25" s="9" t="str">
         <f t="shared" si="11"/>
         <v>したい</v>
       </c>
@@ -3867,7 +3911,7 @@
         <f t="shared" si="12"/>
         <v>しない</v>
       </c>
-      <c r="W25" s="7" t="str">
+      <c r="W25" s="9" t="str">
         <f t="shared" si="12"/>
         <v>しない</v>
       </c>
@@ -3875,21 +3919,26 @@
         <f>_xlfn.CONCAT(T25,"なかった")</f>
         <v>しなかった</v>
       </c>
-      <c r="Y25" s="7" t="str">
+      <c r="Y25" s="9" t="str">
         <f t="shared" si="18"/>
         <v>しなかった</v>
       </c>
       <c r="Z25" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="AA25" s="7" t="s">
+      <c r="AA25" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="AB25" s="7" t="s">
+      <c r="AB25" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="AC25" s="7" t="s">
+      <c r="AC25" s="9" t="s">
         <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.6">
+      <c r="Y28" s="6" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed blank row in excel and added logs to console to troubleshoot
</commit_message>
<xml_diff>
--- a/verbs.xlsx
+++ b/verbs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BradHunt\Documents\japanese-practice\verbs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADF9E73-283B-47DC-B42D-3CD0E1C7B218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34AC361A-5BCD-48F5-A047-511B020D3134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{9921D540-D520-4E46-B0DA-C77DD5C34F2D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="243">
   <si>
     <t>Dictionary</t>
   </si>
@@ -765,9 +765,6 @@
   </si>
   <si>
     <t>およいで</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{566C2546-B21A-4059-8C0C-B1CB9D497EEB}">
-  <dimension ref="A1:AH28"/>
+  <dimension ref="A1:AH25"/>
   <sheetFormatPr defaultRowHeight="17.5" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="12" style="7" bestFit="1" customWidth="1"/>
@@ -3936,11 +3933,6 @@
         <v>147</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.6">
-      <c r="Y28" s="6" t="s">
-        <v>243</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>